<commit_message>
Update: Completed fill in the "No Dependency" in the Dependency column for Nebula and DEET.
Next: Merge them and try to consolidate again to see if it yield better result.
</commit_message>
<xml_diff>
--- a/SWTest/DEET.xlsx
+++ b/SWTest/DEET.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u245231\Quan_Vo\Local_Dev\complete-pandas-tutorial\SWTest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B698A40-956C-491A-8B43-54419AFF0DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D3A056F-DF35-4207-AE05-B2FCC0596232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="2565" windowWidth="16410" windowHeight="18285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DEET" sheetId="2" r:id="rId1"/>
@@ -3575,7 +3575,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="5">
     <dxf>
       <fill>
         <patternFill>
@@ -3620,16 +3620,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3911,22 +3901,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:K504"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.140625" style="32" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="32"/>
-    <col min="3" max="3" width="44.5703125" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.85546875" style="32" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" style="32" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="20.85546875" style="32" customWidth="1"/>
-    <col min="8" max="8" width="15.7109375" style="32" customWidth="1"/>
+    <col min="1" max="1" width="18.109375" style="32" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" style="32"/>
+    <col min="3" max="3" width="44.5546875" style="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.88671875" style="32" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" style="32" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="20.88671875" style="32" customWidth="1"/>
+    <col min="8" max="8" width="15.6640625" style="32" customWidth="1"/>
     <col min="9" max="9" width="29" style="39" customWidth="1"/>
-    <col min="10" max="10" width="39.7109375" style="32" customWidth="1"/>
-    <col min="11" max="11" width="42.7109375" style="32" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="32"/>
+    <col min="10" max="10" width="39.6640625" style="32" customWidth="1"/>
+    <col min="11" max="11" width="42.6640625" style="32" customWidth="1"/>
+    <col min="12" max="16384" width="9.109375" style="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="31" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" s="31" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -3961,7 +3951,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
@@ -3990,7 +3980,7 @@
       </c>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>7</v>
       </c>
@@ -4019,7 +4009,7 @@
       <c r="J3" s="6"/>
       <c r="K3" s="35"/>
     </row>
-    <row r="4" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>7</v>
       </c>
@@ -4048,7 +4038,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
@@ -4075,7 +4065,7 @@
       </c>
       <c r="K5" s="6"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
@@ -4102,7 +4092,7 @@
       <c r="J6" s="6"/>
       <c r="K6" s="35"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>7</v>
       </c>
@@ -4129,7 +4119,7 @@
       <c r="J7" s="6"/>
       <c r="K7" s="35"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>7</v>
       </c>
@@ -4156,7 +4146,7 @@
       <c r="J8" s="6"/>
       <c r="K8" s="35"/>
     </row>
-    <row r="9" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="15" t="s">
         <v>37</v>
       </c>
@@ -4177,7 +4167,7 @@
       <c r="J9" s="12"/>
       <c r="K9" s="12"/>
     </row>
-    <row r="10" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>12</v>
       </c>
@@ -4204,7 +4194,7 @@
       <c r="J10" s="19"/>
       <c r="K10" s="20"/>
     </row>
-    <row r="11" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="15" t="s">
         <v>37</v>
       </c>
@@ -4225,7 +4215,7 @@
       <c r="J11" s="12"/>
       <c r="K11" s="12"/>
     </row>
-    <row r="12" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="15" t="s">
         <v>37</v>
       </c>
@@ -4246,7 +4236,7 @@
       <c r="J12" s="12"/>
       <c r="K12" s="12"/>
     </row>
-    <row r="13" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="15" t="s">
         <v>37</v>
       </c>
@@ -4267,7 +4257,7 @@
       <c r="J13" s="12"/>
       <c r="K13" s="12"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>7</v>
       </c>
@@ -4294,7 +4284,7 @@
       <c r="J14" s="6"/>
       <c r="K14" s="35"/>
     </row>
-    <row r="15" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="15" t="s">
         <v>37</v>
       </c>
@@ -4315,7 +4305,7 @@
       <c r="J15" s="12"/>
       <c r="K15" s="12"/>
     </row>
-    <row r="16" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="15" t="s">
         <v>37</v>
       </c>
@@ -4336,7 +4326,7 @@
       <c r="J16" s="12"/>
       <c r="K16" s="12"/>
     </row>
-    <row r="17" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="15" t="s">
         <v>37</v>
       </c>
@@ -4357,7 +4347,7 @@
       <c r="J17" s="12"/>
       <c r="K17" s="12"/>
     </row>
-    <row r="18" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="15" t="s">
         <v>37</v>
       </c>
@@ -4378,7 +4368,7 @@
       <c r="J18" s="12"/>
       <c r="K18" s="12"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>7</v>
       </c>
@@ -4405,7 +4395,7 @@
       <c r="J19" s="6"/>
       <c r="K19" s="35"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>7</v>
       </c>
@@ -4432,7 +4422,7 @@
       <c r="J20" s="6"/>
       <c r="K20" s="35"/>
     </row>
-    <row r="21" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="15" t="s">
         <v>37</v>
       </c>
@@ -4453,7 +4443,7 @@
       <c r="J21" s="12"/>
       <c r="K21" s="12"/>
     </row>
-    <row r="22" spans="1:11" customFormat="1" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>12</v>
       </c>
@@ -4482,7 +4472,7 @@
       </c>
       <c r="K22" s="20"/>
     </row>
-    <row r="23" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="15" t="s">
         <v>37</v>
       </c>
@@ -4503,7 +4493,7 @@
       <c r="J23" s="12"/>
       <c r="K23" s="12"/>
     </row>
-    <row r="24" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="15" t="s">
         <v>37</v>
       </c>
@@ -4524,7 +4514,7 @@
       <c r="J24" s="12"/>
       <c r="K24" s="12"/>
     </row>
-    <row r="25" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="15" t="s">
         <v>37</v>
       </c>
@@ -4545,7 +4535,7 @@
       <c r="J25" s="12"/>
       <c r="K25" s="12"/>
     </row>
-    <row r="26" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>7</v>
       </c>
@@ -4572,7 +4562,7 @@
       <c r="J26" s="6"/>
       <c r="K26" s="35"/>
     </row>
-    <row r="27" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="15" t="s">
         <v>37</v>
       </c>
@@ -4593,7 +4583,7 @@
       <c r="J27" s="12"/>
       <c r="K27" s="12"/>
     </row>
-    <row r="28" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="15" t="s">
         <v>37</v>
       </c>
@@ -4614,7 +4604,7 @@
       <c r="J28" s="12"/>
       <c r="K28" s="12"/>
     </row>
-    <row r="29" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="15" t="s">
         <v>37</v>
       </c>
@@ -4635,7 +4625,7 @@
       <c r="J29" s="12"/>
       <c r="K29" s="12"/>
     </row>
-    <row r="30" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="15" t="s">
         <v>37</v>
       </c>
@@ -4656,7 +4646,7 @@
       <c r="J30" s="12"/>
       <c r="K30" s="12"/>
     </row>
-    <row r="31" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="15" t="s">
         <v>37</v>
       </c>
@@ -4677,7 +4667,7 @@
       <c r="J31" s="12"/>
       <c r="K31" s="12"/>
     </row>
-    <row r="32" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="15" t="s">
         <v>37</v>
       </c>
@@ -4698,7 +4688,7 @@
       <c r="J32" s="12"/>
       <c r="K32" s="12"/>
     </row>
-    <row r="33" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="15" t="s">
         <v>37</v>
       </c>
@@ -4719,7 +4709,7 @@
       <c r="J33" s="12"/>
       <c r="K33" s="12"/>
     </row>
-    <row r="34" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="15" t="s">
         <v>37</v>
       </c>
@@ -4740,7 +4730,7 @@
       <c r="J34" s="12"/>
       <c r="K34" s="12"/>
     </row>
-    <row r="35" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="15" t="s">
         <v>37</v>
       </c>
@@ -4761,7 +4751,7 @@
       <c r="J35" s="12"/>
       <c r="K35" s="12"/>
     </row>
-    <row r="36" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="15" t="s">
         <v>37</v>
       </c>
@@ -4782,7 +4772,7 @@
       <c r="J36" s="12"/>
       <c r="K36" s="12"/>
     </row>
-    <row r="37" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="15" t="s">
         <v>37</v>
       </c>
@@ -4803,7 +4793,7 @@
       <c r="J37" s="12"/>
       <c r="K37" s="12"/>
     </row>
-    <row r="38" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="15" t="s">
         <v>37</v>
       </c>
@@ -4824,7 +4814,7 @@
       <c r="J38" s="12"/>
       <c r="K38" s="12"/>
     </row>
-    <row r="39" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="15" t="s">
         <v>37</v>
       </c>
@@ -4845,7 +4835,7 @@
       <c r="J39" s="12"/>
       <c r="K39" s="12"/>
     </row>
-    <row r="40" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="15" t="s">
         <v>37</v>
       </c>
@@ -4866,7 +4856,7 @@
       <c r="J40" s="12"/>
       <c r="K40" s="12"/>
     </row>
-    <row r="41" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="15" t="s">
         <v>37</v>
       </c>
@@ -4887,7 +4877,7 @@
       <c r="J41" s="12"/>
       <c r="K41" s="12"/>
     </row>
-    <row r="42" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="15" t="s">
         <v>37</v>
       </c>
@@ -4908,7 +4898,7 @@
       <c r="J42" s="12"/>
       <c r="K42" s="12"/>
     </row>
-    <row r="43" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="15" t="s">
         <v>37</v>
       </c>
@@ -4929,7 +4919,7 @@
       <c r="J43" s="12"/>
       <c r="K43" s="12"/>
     </row>
-    <row r="44" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="15" t="s">
         <v>37</v>
       </c>
@@ -4950,7 +4940,7 @@
       <c r="J44" s="12"/>
       <c r="K44" s="12"/>
     </row>
-    <row r="45" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="15" t="s">
         <v>37</v>
       </c>
@@ -4971,7 +4961,7 @@
       <c r="J45" s="12"/>
       <c r="K45" s="12"/>
     </row>
-    <row r="46" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="15" t="s">
         <v>37</v>
       </c>
@@ -4992,7 +4982,7 @@
       <c r="J46" s="12"/>
       <c r="K46" s="12"/>
     </row>
-    <row r="47" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="15" t="s">
         <v>37</v>
       </c>
@@ -5013,7 +5003,7 @@
       <c r="J47" s="12"/>
       <c r="K47" s="12"/>
     </row>
-    <row r="48" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="15" t="s">
         <v>37</v>
       </c>
@@ -5034,7 +5024,7 @@
       <c r="J48" s="12"/>
       <c r="K48" s="12"/>
     </row>
-    <row r="49" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="15" t="s">
         <v>37</v>
       </c>
@@ -5055,7 +5045,7 @@
       <c r="J49" s="12"/>
       <c r="K49" s="12"/>
     </row>
-    <row r="50" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="15" t="s">
         <v>37</v>
       </c>
@@ -5076,7 +5066,7 @@
       <c r="J50" s="12"/>
       <c r="K50" s="12"/>
     </row>
-    <row r="51" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="15" t="s">
         <v>37</v>
       </c>
@@ -5097,7 +5087,7 @@
       <c r="J51" s="12"/>
       <c r="K51" s="12"/>
     </row>
-    <row r="52" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="15" t="s">
         <v>37</v>
       </c>
@@ -5118,7 +5108,7 @@
       <c r="J52" s="12"/>
       <c r="K52" s="12"/>
     </row>
-    <row r="53" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="15" t="s">
         <v>37</v>
       </c>
@@ -5139,7 +5129,7 @@
       <c r="J53" s="12"/>
       <c r="K53" s="12"/>
     </row>
-    <row r="54" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="15" t="s">
         <v>37</v>
       </c>
@@ -5160,7 +5150,7 @@
       <c r="J54" s="12"/>
       <c r="K54" s="12"/>
     </row>
-    <row r="55" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
         <v>7</v>
       </c>
@@ -5187,7 +5177,7 @@
       <c r="J55" s="6"/>
       <c r="K55" s="35"/>
     </row>
-    <row r="56" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
         <v>7</v>
       </c>
@@ -5214,7 +5204,7 @@
       <c r="J56" s="6"/>
       <c r="K56" s="35"/>
     </row>
-    <row r="57" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
         <v>7</v>
       </c>
@@ -5243,7 +5233,7 @@
       </c>
       <c r="K57" s="5"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
         <v>7</v>
       </c>
@@ -5272,7 +5262,7 @@
       </c>
       <c r="K58" s="5"/>
     </row>
-    <row r="59" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
         <v>7</v>
       </c>
@@ -5299,7 +5289,7 @@
       <c r="J59" s="6"/>
       <c r="K59" s="6"/>
     </row>
-    <row r="60" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
         <v>7</v>
       </c>
@@ -5326,7 +5316,7 @@
       <c r="J60" s="6"/>
       <c r="K60" s="35"/>
     </row>
-    <row r="61" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="15" t="s">
         <v>37</v>
       </c>
@@ -5347,7 +5337,7 @@
       <c r="J61" s="12"/>
       <c r="K61" s="12"/>
     </row>
-    <row r="62" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
         <v>7</v>
       </c>
@@ -5374,7 +5364,7 @@
       <c r="J62" s="6"/>
       <c r="K62" s="35"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
         <v>7</v>
       </c>
@@ -5403,7 +5393,7 @@
       </c>
       <c r="K63" s="35"/>
     </row>
-    <row r="64" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
         <v>7</v>
       </c>
@@ -5434,7 +5424,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="65" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="15" t="s">
         <v>37</v>
       </c>
@@ -5455,7 +5445,7 @@
       <c r="J65" s="12"/>
       <c r="K65" s="12"/>
     </row>
-    <row r="66" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="15" t="s">
         <v>37</v>
       </c>
@@ -5476,7 +5466,7 @@
       <c r="J66" s="12"/>
       <c r="K66" s="12"/>
     </row>
-    <row r="67" spans="1:11" customFormat="1" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
         <v>12</v>
       </c>
@@ -5507,7 +5497,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="43" t="s">
         <v>7</v>
       </c>
@@ -5538,7 +5528,7 @@
       </c>
       <c r="K68" s="43"/>
     </row>
-    <row r="69" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="15" t="s">
         <v>37</v>
       </c>
@@ -5559,7 +5549,7 @@
       <c r="J69" s="12"/>
       <c r="K69" s="12"/>
     </row>
-    <row r="70" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="15" t="s">
         <v>37</v>
       </c>
@@ -5580,7 +5570,7 @@
       <c r="J70" s="12"/>
       <c r="K70" s="12"/>
     </row>
-    <row r="71" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
         <v>12</v>
       </c>
@@ -5609,7 +5599,7 @@
       </c>
       <c r="K71" s="20"/>
     </row>
-    <row r="72" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="43" t="s">
         <v>7</v>
       </c>
@@ -5640,7 +5630,7 @@
       </c>
       <c r="K72" s="48"/>
     </row>
-    <row r="73" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
         <v>12</v>
       </c>
@@ -5669,7 +5659,7 @@
       </c>
       <c r="K73" s="20"/>
     </row>
-    <row r="74" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
         <v>12</v>
       </c>
@@ -5698,7 +5688,7 @@
       </c>
       <c r="K74" s="20"/>
     </row>
-    <row r="75" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
         <v>7</v>
       </c>
@@ -5725,7 +5715,7 @@
       <c r="J75" s="6"/>
       <c r="K75" s="35"/>
     </row>
-    <row r="76" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="15" t="s">
         <v>37</v>
       </c>
@@ -5746,7 +5736,7 @@
       <c r="J76" s="12"/>
       <c r="K76" s="12"/>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
         <v>7</v>
       </c>
@@ -5775,7 +5765,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
         <v>7</v>
       </c>
@@ -5804,7 +5794,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="79" spans="1:11" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
         <v>12</v>
       </c>
@@ -5833,7 +5823,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="43" t="s">
         <v>7</v>
       </c>
@@ -5862,7 +5852,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
         <v>7</v>
       </c>
@@ -5891,7 +5881,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="43" t="s">
         <v>7</v>
       </c>
@@ -5920,7 +5910,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="83" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="15" t="s">
         <v>37</v>
       </c>
@@ -5941,7 +5931,7 @@
       <c r="J83" s="12"/>
       <c r="K83" s="12"/>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
         <v>7</v>
       </c>
@@ -5968,7 +5958,7 @@
       <c r="J84" s="6"/>
       <c r="K84" s="5"/>
     </row>
-    <row r="85" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="15" t="s">
         <v>37</v>
       </c>
@@ -5989,7 +5979,7 @@
       <c r="J85" s="12"/>
       <c r="K85" s="12"/>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="43" t="s">
         <v>7</v>
       </c>
@@ -6016,7 +6006,7 @@
       <c r="J86" s="48"/>
       <c r="K86" s="50"/>
     </row>
-    <row r="87" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="5" t="s">
         <v>12</v>
       </c>
@@ -6045,7 +6035,7 @@
       </c>
       <c r="K87" s="19"/>
     </row>
-    <row r="88" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="5" t="s">
         <v>7</v>
       </c>
@@ -6076,7 +6066,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="89" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="15" t="s">
         <v>37</v>
       </c>
@@ -6097,7 +6087,7 @@
       <c r="J89" s="12"/>
       <c r="K89" s="12"/>
     </row>
-    <row r="90" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="15" t="s">
         <v>37</v>
       </c>
@@ -6118,7 +6108,7 @@
       <c r="J90" s="12"/>
       <c r="K90" s="12"/>
     </row>
-    <row r="91" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:11" ht="69" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
         <v>7</v>
       </c>
@@ -6149,7 +6139,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="5" t="s">
         <v>7</v>
       </c>
@@ -6176,7 +6166,7 @@
       <c r="J92" s="6"/>
       <c r="K92" s="5"/>
     </row>
-    <row r="93" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
         <v>7</v>
       </c>
@@ -6205,7 +6195,7 @@
       </c>
       <c r="K93" s="6"/>
     </row>
-    <row r="94" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" s="15" t="s">
         <v>37</v>
       </c>
@@ -6226,7 +6216,7 @@
       <c r="J94" s="12"/>
       <c r="K94" s="12"/>
     </row>
-    <row r="95" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="15" t="s">
         <v>37</v>
       </c>
@@ -6247,7 +6237,7 @@
       <c r="J95" s="12"/>
       <c r="K95" s="12"/>
     </row>
-    <row r="96" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="15" t="s">
         <v>37</v>
       </c>
@@ -6268,7 +6258,7 @@
       <c r="J96" s="12"/>
       <c r="K96" s="12"/>
     </row>
-    <row r="97" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="5" t="s">
         <v>7</v>
       </c>
@@ -6301,7 +6291,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="98" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
         <v>12</v>
       </c>
@@ -6330,7 +6320,7 @@
       </c>
       <c r="K98" s="12"/>
     </row>
-    <row r="99" spans="1:11" customFormat="1" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:11" customFormat="1" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
         <v>12</v>
       </c>
@@ -6359,7 +6349,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="100" spans="1:11" customFormat="1" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:11" customFormat="1" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="5" t="s">
         <v>12</v>
       </c>
@@ -6388,7 +6378,7 @@
       </c>
       <c r="K100" s="19"/>
     </row>
-    <row r="101" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
         <v>12</v>
       </c>
@@ -6417,7 +6407,7 @@
       </c>
       <c r="K101" s="19"/>
     </row>
-    <row r="102" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
         <v>12</v>
       </c>
@@ -6446,7 +6436,7 @@
       </c>
       <c r="K102" s="19"/>
     </row>
-    <row r="103" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="5" t="s">
         <v>12</v>
       </c>
@@ -6475,7 +6465,7 @@
       </c>
       <c r="K103" s="19"/>
     </row>
-    <row r="104" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="5" t="s">
         <v>12</v>
       </c>
@@ -6504,7 +6494,7 @@
       </c>
       <c r="K104" s="19"/>
     </row>
-    <row r="105" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="5" t="s">
         <v>12</v>
       </c>
@@ -6533,7 +6523,7 @@
       </c>
       <c r="K105" s="19"/>
     </row>
-    <row r="106" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" s="5" t="s">
         <v>12</v>
       </c>
@@ -6562,7 +6552,7 @@
       </c>
       <c r="K106" s="19"/>
     </row>
-    <row r="107" spans="1:11" customFormat="1" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:11" customFormat="1" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="5" t="s">
         <v>12</v>
       </c>
@@ -6591,7 +6581,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="108" spans="1:11" customFormat="1" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:11" customFormat="1" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="5" t="s">
         <v>12</v>
       </c>
@@ -6620,7 +6610,7 @@
       </c>
       <c r="K108" s="19"/>
     </row>
-    <row r="109" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="5" t="s">
         <v>12</v>
       </c>
@@ -6647,7 +6637,7 @@
       <c r="J109" s="19"/>
       <c r="K109" s="20"/>
     </row>
-    <row r="110" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
         <v>12</v>
       </c>
@@ -6674,7 +6664,7 @@
       <c r="J110" s="19"/>
       <c r="K110" s="19"/>
     </row>
-    <row r="111" spans="1:11" customFormat="1" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="5" t="s">
         <v>12</v>
       </c>
@@ -6703,7 +6693,7 @@
       </c>
       <c r="K111" s="19"/>
     </row>
-    <row r="112" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="15" t="s">
         <v>37</v>
       </c>
@@ -6724,7 +6714,7 @@
       <c r="J112" s="12"/>
       <c r="K112" s="12"/>
     </row>
-    <row r="113" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="15" t="s">
         <v>37</v>
       </c>
@@ -6745,7 +6735,7 @@
       <c r="J113" s="12"/>
       <c r="K113" s="12"/>
     </row>
-    <row r="114" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" s="15" t="s">
         <v>37</v>
       </c>
@@ -6766,7 +6756,7 @@
       <c r="J114" s="12"/>
       <c r="K114" s="12"/>
     </row>
-    <row r="115" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="15" t="s">
         <v>37</v>
       </c>
@@ -6787,7 +6777,7 @@
       <c r="J115" s="12"/>
       <c r="K115" s="12"/>
     </row>
-    <row r="116" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" s="15" t="s">
         <v>37</v>
       </c>
@@ -6808,7 +6798,7 @@
       <c r="J116" s="12"/>
       <c r="K116" s="12"/>
     </row>
-    <row r="117" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="15" t="s">
         <v>37</v>
       </c>
@@ -6829,7 +6819,7 @@
       <c r="J117" s="12"/>
       <c r="K117" s="12"/>
     </row>
-    <row r="118" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="5" t="s">
         <v>12</v>
       </c>
@@ -6856,7 +6846,7 @@
       <c r="J118" s="19"/>
       <c r="K118" s="20"/>
     </row>
-    <row r="119" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="15" t="s">
         <v>37</v>
       </c>
@@ -6877,7 +6867,7 @@
       <c r="J119" s="12"/>
       <c r="K119" s="12"/>
     </row>
-    <row r="120" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="5" t="s">
         <v>12</v>
       </c>
@@ -6906,7 +6896,7 @@
       </c>
       <c r="K120" s="12"/>
     </row>
-    <row r="121" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="5" t="s">
         <v>7</v>
       </c>
@@ -6935,7 +6925,7 @@
       </c>
       <c r="K121" s="5"/>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="5" t="s">
         <v>7</v>
       </c>
@@ -6962,7 +6952,7 @@
       </c>
       <c r="K122" s="5"/>
     </row>
-    <row r="123" spans="1:11" customFormat="1" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="5" t="s">
         <v>12</v>
       </c>
@@ -6993,7 +6983,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="124" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="5" t="s">
         <v>7</v>
       </c>
@@ -7026,7 +7016,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="125" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="15" t="s">
         <v>37</v>
       </c>
@@ -7047,7 +7037,7 @@
       <c r="J125" s="12"/>
       <c r="K125" s="12"/>
     </row>
-    <row r="126" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="15" t="s">
         <v>37</v>
       </c>
@@ -7068,7 +7058,7 @@
       <c r="J126" s="12"/>
       <c r="K126" s="12"/>
     </row>
-    <row r="127" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="15" t="s">
         <v>37</v>
       </c>
@@ -7089,7 +7079,7 @@
       <c r="J127" s="12"/>
       <c r="K127" s="12"/>
     </row>
-    <row r="128" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="5" t="s">
         <v>12</v>
       </c>
@@ -7116,7 +7106,7 @@
       <c r="J128" s="12"/>
       <c r="K128" s="19"/>
     </row>
-    <row r="129" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="5" t="s">
         <v>7</v>
       </c>
@@ -7145,7 +7135,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="130" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="15" t="s">
         <v>37</v>
       </c>
@@ -7166,7 +7156,7 @@
       <c r="J130" s="12"/>
       <c r="K130" s="12"/>
     </row>
-    <row r="131" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="15" t="s">
         <v>37</v>
       </c>
@@ -7187,7 +7177,7 @@
       <c r="J131" s="12"/>
       <c r="K131" s="12"/>
     </row>
-    <row r="132" spans="1:11" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="5" t="s">
         <v>12</v>
       </c>
@@ -7216,7 +7206,7 @@
       </c>
       <c r="K132" s="12"/>
     </row>
-    <row r="133" spans="1:11" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" s="5" t="s">
         <v>12</v>
       </c>
@@ -7245,7 +7235,7 @@
       </c>
       <c r="K133" s="19"/>
     </row>
-    <row r="134" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="5" t="s">
         <v>7</v>
       </c>
@@ -7274,7 +7264,7 @@
       </c>
       <c r="K134" s="5"/>
     </row>
-    <row r="135" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:11" ht="69" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="5" t="s">
         <v>7</v>
       </c>
@@ -7301,7 +7291,7 @@
       </c>
       <c r="K135" s="6"/>
     </row>
-    <row r="136" spans="1:11" customFormat="1" ht="26.25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="5" t="s">
         <v>12</v>
       </c>
@@ -7328,7 +7318,7 @@
       <c r="J136" s="19"/>
       <c r="K136" s="12"/>
     </row>
-    <row r="137" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:11" ht="69" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" s="5" t="s">
         <v>7</v>
       </c>
@@ -7355,7 +7345,7 @@
       </c>
       <c r="K137" s="6"/>
     </row>
-    <row r="138" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:11" ht="69" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="5" t="s">
         <v>7</v>
       </c>
@@ -7382,7 +7372,7 @@
       </c>
       <c r="K138" s="6"/>
     </row>
-    <row r="139" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:11" ht="69" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" s="5" t="s">
         <v>7</v>
       </c>
@@ -7409,7 +7399,7 @@
       </c>
       <c r="K139" s="5"/>
     </row>
-    <row r="140" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A140" s="15" t="s">
         <v>16</v>
       </c>
@@ -7434,7 +7424,7 @@
       <c r="J140" s="5"/>
       <c r="K140" s="5"/>
     </row>
-    <row r="141" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A141" s="15" t="s">
         <v>16</v>
       </c>
@@ -7459,7 +7449,7 @@
       <c r="J141" s="5"/>
       <c r="K141" s="5"/>
     </row>
-    <row r="142" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" s="15" t="s">
         <v>37</v>
       </c>
@@ -7480,7 +7470,7 @@
       <c r="J142" s="12"/>
       <c r="K142" s="12"/>
     </row>
-    <row r="143" spans="1:11" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" s="5" t="s">
         <v>12</v>
       </c>
@@ -7509,7 +7499,7 @@
       </c>
       <c r="K143" s="19"/>
     </row>
-    <row r="144" spans="1:11" customFormat="1" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:11" customFormat="1" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" s="5" t="s">
         <v>12</v>
       </c>
@@ -7540,7 +7530,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="145" spans="1:11" customFormat="1" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:11" customFormat="1" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" s="5" t="s">
         <v>12</v>
       </c>
@@ -7571,7 +7561,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="146" spans="1:11" customFormat="1" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:11" customFormat="1" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" s="5" t="s">
         <v>12</v>
       </c>
@@ -7602,7 +7592,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="147" spans="1:11" customFormat="1" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:11" customFormat="1" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="5" t="s">
         <v>12</v>
       </c>
@@ -7633,7 +7623,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="148" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="15" t="s">
         <v>37</v>
       </c>
@@ -7654,7 +7644,7 @@
       <c r="J148" s="12"/>
       <c r="K148" s="12"/>
     </row>
-    <row r="149" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A149" s="15" t="s">
         <v>16</v>
       </c>
@@ -7679,7 +7669,7 @@
       <c r="J149" s="5"/>
       <c r="K149" s="5"/>
     </row>
-    <row r="150" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A150" s="15" t="s">
         <v>16</v>
       </c>
@@ -7704,7 +7694,7 @@
       <c r="J150" s="5"/>
       <c r="K150" s="5"/>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" s="15" t="s">
         <v>16</v>
       </c>
@@ -7729,7 +7719,7 @@
       <c r="J151" s="5"/>
       <c r="K151" s="5"/>
     </row>
-    <row r="152" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" s="15" t="s">
         <v>16</v>
       </c>
@@ -7758,7 +7748,7 @@
       </c>
       <c r="K152" s="5"/>
     </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" s="5" t="s">
         <v>16</v>
       </c>
@@ -7785,7 +7775,7 @@
       </c>
       <c r="K153" s="5"/>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="5" t="s">
         <v>16</v>
       </c>
@@ -7810,7 +7800,7 @@
       <c r="J154" s="5"/>
       <c r="K154" s="5"/>
     </row>
-    <row r="155" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="15" t="s">
         <v>37</v>
       </c>
@@ -7831,7 +7821,7 @@
       <c r="J155" s="12"/>
       <c r="K155" s="12"/>
     </row>
-    <row r="156" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" s="15" t="s">
         <v>37</v>
       </c>
@@ -7852,7 +7842,7 @@
       <c r="J156" s="12"/>
       <c r="K156" s="12"/>
     </row>
-    <row r="157" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" s="15" t="s">
         <v>37</v>
       </c>
@@ -7873,7 +7863,7 @@
       <c r="J157" s="12"/>
       <c r="K157" s="12"/>
     </row>
-    <row r="158" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" s="15" t="s">
         <v>37</v>
       </c>
@@ -7894,7 +7884,7 @@
       <c r="J158" s="12"/>
       <c r="K158" s="12"/>
     </row>
-    <row r="159" spans="1:11" ht="0.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:11" ht="0.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" s="5" t="s">
         <v>16</v>
       </c>
@@ -7921,7 +7911,7 @@
       <c r="J159" s="5"/>
       <c r="K159" s="5"/>
     </row>
-    <row r="160" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" s="15" t="s">
         <v>37</v>
       </c>
@@ -7942,7 +7932,7 @@
       <c r="J160" s="12"/>
       <c r="K160" s="12"/>
     </row>
-    <row r="161" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" s="15" t="s">
         <v>37</v>
       </c>
@@ -7963,7 +7953,7 @@
       <c r="J161" s="12"/>
       <c r="K161" s="12"/>
     </row>
-    <row r="162" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" s="15" t="s">
         <v>37</v>
       </c>
@@ -7984,7 +7974,7 @@
       <c r="J162" s="12"/>
       <c r="K162" s="12"/>
     </row>
-    <row r="163" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" s="15" t="s">
         <v>37</v>
       </c>
@@ -8005,7 +7995,7 @@
       <c r="J163" s="12"/>
       <c r="K163" s="12"/>
     </row>
-    <row r="164" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" s="15" t="s">
         <v>37</v>
       </c>
@@ -8026,7 +8016,7 @@
       <c r="J164" s="12"/>
       <c r="K164" s="12"/>
     </row>
-    <row r="165" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" s="15" t="s">
         <v>37</v>
       </c>
@@ -8047,7 +8037,7 @@
       <c r="J165" s="12"/>
       <c r="K165" s="12"/>
     </row>
-    <row r="166" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" s="15" t="s">
         <v>37</v>
       </c>
@@ -8068,7 +8058,7 @@
       <c r="J166" s="12"/>
       <c r="K166" s="12"/>
     </row>
-    <row r="167" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" s="15" t="s">
         <v>37</v>
       </c>
@@ -8089,7 +8079,7 @@
       <c r="J167" s="12"/>
       <c r="K167" s="12"/>
     </row>
-    <row r="168" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" s="15" t="s">
         <v>37</v>
       </c>
@@ -8110,7 +8100,7 @@
       <c r="J168" s="12"/>
       <c r="K168" s="12"/>
     </row>
-    <row r="169" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" s="15" t="s">
         <v>37</v>
       </c>
@@ -8131,7 +8121,7 @@
       <c r="J169" s="12"/>
       <c r="K169" s="12"/>
     </row>
-    <row r="170" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" s="15" t="s">
         <v>37</v>
       </c>
@@ -8152,7 +8142,7 @@
       <c r="J170" s="12"/>
       <c r="K170" s="12"/>
     </row>
-    <row r="171" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" s="15" t="s">
         <v>37</v>
       </c>
@@ -8173,7 +8163,7 @@
       <c r="J171" s="12"/>
       <c r="K171" s="12"/>
     </row>
-    <row r="172" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" s="15" t="s">
         <v>37</v>
       </c>
@@ -8194,7 +8184,7 @@
       <c r="J172" s="12"/>
       <c r="K172" s="12"/>
     </row>
-    <row r="173" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" s="15" t="s">
         <v>37</v>
       </c>
@@ -8215,7 +8205,7 @@
       <c r="J173" s="12"/>
       <c r="K173" s="12"/>
     </row>
-    <row r="174" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" s="15" t="s">
         <v>37</v>
       </c>
@@ -8236,7 +8226,7 @@
       <c r="J174" s="12"/>
       <c r="K174" s="12"/>
     </row>
-    <row r="175" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" s="15" t="s">
         <v>37</v>
       </c>
@@ -8257,7 +8247,7 @@
       <c r="J175" s="12"/>
       <c r="K175" s="12"/>
     </row>
-    <row r="176" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" s="15" t="s">
         <v>37</v>
       </c>
@@ -8278,7 +8268,7 @@
       <c r="J176" s="12"/>
       <c r="K176" s="12"/>
     </row>
-    <row r="177" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" s="15" t="s">
         <v>37</v>
       </c>
@@ -8299,7 +8289,7 @@
       <c r="J177" s="12"/>
       <c r="K177" s="12"/>
     </row>
-    <row r="178" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" s="15" t="s">
         <v>37</v>
       </c>
@@ -8320,7 +8310,7 @@
       <c r="J178" s="12"/>
       <c r="K178" s="12"/>
     </row>
-    <row r="179" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" s="15" t="s">
         <v>37</v>
       </c>
@@ -8341,7 +8331,7 @@
       <c r="J179" s="12"/>
       <c r="K179" s="12"/>
     </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" s="5" t="s">
         <v>16</v>
       </c>
@@ -8366,7 +8356,7 @@
       <c r="J180" s="5"/>
       <c r="K180" s="5"/>
     </row>
-    <row r="181" spans="1:11" ht="0.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:11" ht="0.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A181" s="5" t="s">
         <v>16</v>
       </c>
@@ -8393,7 +8383,7 @@
       <c r="J181" s="5"/>
       <c r="K181" s="5"/>
     </row>
-    <row r="182" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" s="5" t="s">
         <v>16</v>
       </c>
@@ -8420,7 +8410,7 @@
       <c r="J182" s="5"/>
       <c r="K182" s="5"/>
     </row>
-    <row r="183" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" s="15" t="s">
         <v>37</v>
       </c>
@@ -8441,7 +8431,7 @@
       <c r="J183" s="12"/>
       <c r="K183" s="12"/>
     </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" s="5" t="s">
         <v>16</v>
       </c>
@@ -8468,7 +8458,7 @@
       <c r="J184" s="5"/>
       <c r="K184" s="5"/>
     </row>
-    <row r="185" spans="1:11" ht="1.1499999999999999" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:11" ht="1.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A185" s="5" t="s">
         <v>16</v>
       </c>
@@ -8495,7 +8485,7 @@
       <c r="J185" s="5"/>
       <c r="K185" s="5"/>
     </row>
-    <row r="186" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" s="15" t="s">
         <v>37</v>
       </c>
@@ -8516,7 +8506,7 @@
       <c r="J186" s="12"/>
       <c r="K186" s="12"/>
     </row>
-    <row r="187" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" s="15" t="s">
         <v>37</v>
       </c>
@@ -8537,7 +8527,7 @@
       <c r="J187" s="12"/>
       <c r="K187" s="12"/>
     </row>
-    <row r="188" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" s="15" t="s">
         <v>37</v>
       </c>
@@ -8558,7 +8548,7 @@
       <c r="J188" s="12"/>
       <c r="K188" s="12"/>
     </row>
-    <row r="189" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" s="15" t="s">
         <v>37</v>
       </c>
@@ -8579,7 +8569,7 @@
       <c r="J189" s="12"/>
       <c r="K189" s="12"/>
     </row>
-    <row r="190" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" s="15" t="s">
         <v>37</v>
       </c>
@@ -8600,7 +8590,7 @@
       <c r="J190" s="12"/>
       <c r="K190" s="12"/>
     </row>
-    <row r="191" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" s="15" t="s">
         <v>37</v>
       </c>
@@ -8621,7 +8611,7 @@
       <c r="J191" s="12"/>
       <c r="K191" s="12"/>
     </row>
-    <row r="192" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" s="15" t="s">
         <v>37</v>
       </c>
@@ -8642,7 +8632,7 @@
       <c r="J192" s="12"/>
       <c r="K192" s="12"/>
     </row>
-    <row r="193" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" s="15" t="s">
         <v>37</v>
       </c>
@@ -8663,7 +8653,7 @@
       <c r="J193" s="12"/>
       <c r="K193" s="12"/>
     </row>
-    <row r="194" spans="1:11" ht="0.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:11" ht="0.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A194" s="5" t="s">
         <v>16</v>
       </c>
@@ -8688,7 +8678,7 @@
       <c r="J194" s="5"/>
       <c r="K194" s="5"/>
     </row>
-    <row r="195" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" s="15" t="s">
         <v>37</v>
       </c>
@@ -8709,7 +8699,7 @@
       <c r="J195" s="12"/>
       <c r="K195" s="12"/>
     </row>
-    <row r="196" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" s="15" t="s">
         <v>37</v>
       </c>
@@ -8730,7 +8720,7 @@
       <c r="J196" s="12"/>
       <c r="K196" s="12"/>
     </row>
-    <row r="197" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" s="15" t="s">
         <v>37</v>
       </c>
@@ -8751,7 +8741,7 @@
       <c r="J197" s="12"/>
       <c r="K197" s="12"/>
     </row>
-    <row r="198" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" s="15" t="s">
         <v>37</v>
       </c>
@@ -8772,7 +8762,7 @@
       <c r="J198" s="12"/>
       <c r="K198" s="12"/>
     </row>
-    <row r="199" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" s="15" t="s">
         <v>37</v>
       </c>
@@ -8793,7 +8783,7 @@
       <c r="J199" s="12"/>
       <c r="K199" s="12"/>
     </row>
-    <row r="200" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" s="15" t="s">
         <v>37</v>
       </c>
@@ -8814,7 +8804,7 @@
       <c r="J200" s="12"/>
       <c r="K200" s="12"/>
     </row>
-    <row r="201" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" s="15" t="s">
         <v>37</v>
       </c>
@@ -8835,7 +8825,7 @@
       <c r="J201" s="12"/>
       <c r="K201" s="12"/>
     </row>
-    <row r="202" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" s="15" t="s">
         <v>37</v>
       </c>
@@ -8856,7 +8846,7 @@
       <c r="J202" s="12"/>
       <c r="K202" s="12"/>
     </row>
-    <row r="203" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" s="15" t="s">
         <v>37</v>
       </c>
@@ -8877,7 +8867,7 @@
       <c r="J203" s="12"/>
       <c r="K203" s="12"/>
     </row>
-    <row r="204" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" s="15" t="s">
         <v>37</v>
       </c>
@@ -8898,7 +8888,7 @@
       <c r="J204" s="12"/>
       <c r="K204" s="12"/>
     </row>
-    <row r="205" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" s="15" t="s">
         <v>37</v>
       </c>
@@ -8919,7 +8909,7 @@
       <c r="J205" s="12"/>
       <c r="K205" s="12"/>
     </row>
-    <row r="206" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" s="5" t="s">
         <v>16</v>
       </c>
@@ -8946,7 +8936,7 @@
       <c r="J206" s="5"/>
       <c r="K206" s="5"/>
     </row>
-    <row r="207" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" s="5" t="s">
         <v>16</v>
       </c>
@@ -8973,7 +8963,7 @@
       <c r="J207" s="5"/>
       <c r="K207" s="5"/>
     </row>
-    <row r="208" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" s="5" t="s">
         <v>16</v>
       </c>
@@ -9000,7 +8990,7 @@
       <c r="J208" s="5"/>
       <c r="K208" s="5"/>
     </row>
-    <row r="209" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" s="5" t="s">
         <v>16</v>
       </c>
@@ -9025,7 +9015,7 @@
       <c r="J209" s="5"/>
       <c r="K209" s="5"/>
     </row>
-    <row r="210" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" s="15" t="s">
         <v>37</v>
       </c>
@@ -9046,7 +9036,7 @@
       <c r="J210" s="12"/>
       <c r="K210" s="12"/>
     </row>
-    <row r="211" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" s="5" t="s">
         <v>16</v>
       </c>
@@ -9071,7 +9061,7 @@
       <c r="J211" s="5"/>
       <c r="K211" s="5"/>
     </row>
-    <row r="212" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212" s="15" t="s">
         <v>37</v>
       </c>
@@ -9092,7 +9082,7 @@
       <c r="J212" s="12"/>
       <c r="K212" s="12"/>
     </row>
-    <row r="213" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" s="15" t="s">
         <v>37</v>
       </c>
@@ -9113,7 +9103,7 @@
       <c r="J213" s="12"/>
       <c r="K213" s="12"/>
     </row>
-    <row r="214" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" s="15" t="s">
         <v>37</v>
       </c>
@@ -9134,7 +9124,7 @@
       <c r="J214" s="12"/>
       <c r="K214" s="12"/>
     </row>
-    <row r="215" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" s="5" t="s">
         <v>16</v>
       </c>
@@ -9159,7 +9149,7 @@
       <c r="J215" s="5"/>
       <c r="K215" s="5"/>
     </row>
-    <row r="216" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" s="5" t="s">
         <v>16</v>
       </c>
@@ -9184,7 +9174,7 @@
       <c r="J216" s="5"/>
       <c r="K216" s="5"/>
     </row>
-    <row r="217" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" s="15" t="s">
         <v>37</v>
       </c>
@@ -9205,7 +9195,7 @@
       <c r="J217" s="12"/>
       <c r="K217" s="12"/>
     </row>
-    <row r="218" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" s="15" t="s">
         <v>37</v>
       </c>
@@ -9226,7 +9216,7 @@
       <c r="J218" s="12"/>
       <c r="K218" s="12"/>
     </row>
-    <row r="219" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" s="15" t="s">
         <v>37</v>
       </c>
@@ -9247,7 +9237,7 @@
       <c r="J219" s="12"/>
       <c r="K219" s="12"/>
     </row>
-    <row r="220" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220" s="15" t="s">
         <v>37</v>
       </c>
@@ -9268,7 +9258,7 @@
       <c r="J220" s="12"/>
       <c r="K220" s="12"/>
     </row>
-    <row r="221" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" s="5" t="s">
         <v>16</v>
       </c>
@@ -9295,7 +9285,7 @@
       <c r="J221" s="5"/>
       <c r="K221" s="5"/>
     </row>
-    <row r="222" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" s="5" t="s">
         <v>16</v>
       </c>
@@ -9322,7 +9312,7 @@
       <c r="J222" s="5"/>
       <c r="K222" s="5"/>
     </row>
-    <row r="223" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223" s="15" t="s">
         <v>37</v>
       </c>
@@ -9343,7 +9333,7 @@
       <c r="J223" s="12"/>
       <c r="K223" s="12"/>
     </row>
-    <row r="224" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224" s="15" t="s">
         <v>37</v>
       </c>
@@ -9364,7 +9354,7 @@
       <c r="J224" s="12"/>
       <c r="K224" s="12"/>
     </row>
-    <row r="225" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" s="15" t="s">
         <v>37</v>
       </c>
@@ -9385,7 +9375,7 @@
       <c r="J225" s="12"/>
       <c r="K225" s="12"/>
     </row>
-    <row r="226" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226" s="15" t="s">
         <v>37</v>
       </c>
@@ -9406,7 +9396,7 @@
       <c r="J226" s="12"/>
       <c r="K226" s="12"/>
     </row>
-    <row r="227" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227" s="15" t="s">
         <v>37</v>
       </c>
@@ -9427,7 +9417,7 @@
       <c r="J227" s="12"/>
       <c r="K227" s="12"/>
     </row>
-    <row r="228" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" s="15" t="s">
         <v>37</v>
       </c>
@@ -9448,7 +9438,7 @@
       <c r="J228" s="12"/>
       <c r="K228" s="12"/>
     </row>
-    <row r="229" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" s="5" t="s">
         <v>16</v>
       </c>
@@ -9475,7 +9465,7 @@
       <c r="J229" s="5"/>
       <c r="K229" s="5"/>
     </row>
-    <row r="230" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230" s="5" t="s">
         <v>16</v>
       </c>
@@ -9502,7 +9492,7 @@
       <c r="J230" s="5"/>
       <c r="K230" s="5"/>
     </row>
-    <row r="231" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" s="5" t="s">
         <v>16</v>
       </c>
@@ -9527,7 +9517,7 @@
       <c r="J231" s="5"/>
       <c r="K231" s="5"/>
     </row>
-    <row r="232" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232" s="15" t="s">
         <v>37</v>
       </c>
@@ -9548,7 +9538,7 @@
       <c r="J232" s="12"/>
       <c r="K232" s="12"/>
     </row>
-    <row r="233" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233" s="15" t="s">
         <v>37</v>
       </c>
@@ -9569,7 +9559,7 @@
       <c r="J233" s="12"/>
       <c r="K233" s="12"/>
     </row>
-    <row r="234" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234" s="15" t="s">
         <v>37</v>
       </c>
@@ -9590,7 +9580,7 @@
       <c r="J234" s="12"/>
       <c r="K234" s="12"/>
     </row>
-    <row r="235" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" s="15" t="s">
         <v>37</v>
       </c>
@@ -9611,7 +9601,7 @@
       <c r="J235" s="12"/>
       <c r="K235" s="12"/>
     </row>
-    <row r="236" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236" s="15" t="s">
         <v>37</v>
       </c>
@@ -9632,7 +9622,7 @@
       <c r="J236" s="12"/>
       <c r="K236" s="12"/>
     </row>
-    <row r="237" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237" s="15" t="s">
         <v>37</v>
       </c>
@@ -9653,7 +9643,7 @@
       <c r="J237" s="12"/>
       <c r="K237" s="12"/>
     </row>
-    <row r="238" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" s="15" t="s">
         <v>37</v>
       </c>
@@ -9674,7 +9664,7 @@
       <c r="J238" s="12"/>
       <c r="K238" s="12"/>
     </row>
-    <row r="239" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239" s="15" t="s">
         <v>37</v>
       </c>
@@ -9695,7 +9685,7 @@
       <c r="J239" s="12"/>
       <c r="K239" s="12"/>
     </row>
-    <row r="240" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240" s="15" t="s">
         <v>37</v>
       </c>
@@ -9716,7 +9706,7 @@
       <c r="J240" s="12"/>
       <c r="K240" s="12"/>
     </row>
-    <row r="241" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241" s="15" t="s">
         <v>37</v>
       </c>
@@ -9737,7 +9727,7 @@
       <c r="J241" s="12"/>
       <c r="K241" s="12"/>
     </row>
-    <row r="242" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" s="15" t="s">
         <v>37</v>
       </c>
@@ -9758,7 +9748,7 @@
       <c r="J242" s="12"/>
       <c r="K242" s="12"/>
     </row>
-    <row r="243" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243" s="15" t="s">
         <v>37</v>
       </c>
@@ -9779,7 +9769,7 @@
       <c r="J243" s="12"/>
       <c r="K243" s="12"/>
     </row>
-    <row r="244" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" s="15" t="s">
         <v>37</v>
       </c>
@@ -9800,7 +9790,7 @@
       <c r="J244" s="12"/>
       <c r="K244" s="12"/>
     </row>
-    <row r="245" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245" s="15" t="s">
         <v>37</v>
       </c>
@@ -9821,7 +9811,7 @@
       <c r="J245" s="12"/>
       <c r="K245" s="12"/>
     </row>
-    <row r="246" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246" s="15" t="s">
         <v>37</v>
       </c>
@@ -9842,7 +9832,7 @@
       <c r="J246" s="12"/>
       <c r="K246" s="12"/>
     </row>
-    <row r="247" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247" s="15" t="s">
         <v>37</v>
       </c>
@@ -9863,7 +9853,7 @@
       <c r="J247" s="12"/>
       <c r="K247" s="12"/>
     </row>
-    <row r="248" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248" s="15" t="s">
         <v>37</v>
       </c>
@@ -9884,7 +9874,7 @@
       <c r="J248" s="12"/>
       <c r="K248" s="12"/>
     </row>
-    <row r="249" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" s="15" t="s">
         <v>37</v>
       </c>
@@ -9905,7 +9895,7 @@
       <c r="J249" s="12"/>
       <c r="K249" s="12"/>
     </row>
-    <row r="250" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" s="15" t="s">
         <v>37</v>
       </c>
@@ -9926,7 +9916,7 @@
       <c r="J250" s="12"/>
       <c r="K250" s="12"/>
     </row>
-    <row r="251" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" s="15" t="s">
         <v>37</v>
       </c>
@@ -9947,7 +9937,7 @@
       <c r="J251" s="12"/>
       <c r="K251" s="12"/>
     </row>
-    <row r="252" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252" s="15" t="s">
         <v>37</v>
       </c>
@@ -9968,7 +9958,7 @@
       <c r="J252" s="12"/>
       <c r="K252" s="12"/>
     </row>
-    <row r="253" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253" s="15" t="s">
         <v>37</v>
       </c>
@@ -9989,7 +9979,7 @@
       <c r="J253" s="12"/>
       <c r="K253" s="12"/>
     </row>
-    <row r="254" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" s="15" t="s">
         <v>37</v>
       </c>
@@ -10010,7 +10000,7 @@
       <c r="J254" s="12"/>
       <c r="K254" s="12"/>
     </row>
-    <row r="255" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255" s="15" t="s">
         <v>37</v>
       </c>
@@ -10031,7 +10021,7 @@
       <c r="J255" s="12"/>
       <c r="K255" s="12"/>
     </row>
-    <row r="256" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256" s="15" t="s">
         <v>37</v>
       </c>
@@ -10052,7 +10042,7 @@
       <c r="J256" s="12"/>
       <c r="K256" s="12"/>
     </row>
-    <row r="257" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" s="15" t="s">
         <v>37</v>
       </c>
@@ -10073,7 +10063,7 @@
       <c r="J257" s="12"/>
       <c r="K257" s="12"/>
     </row>
-    <row r="258" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A258" s="15" t="s">
         <v>37</v>
       </c>
@@ -10094,7 +10084,7 @@
       <c r="J258" s="12"/>
       <c r="K258" s="12"/>
     </row>
-    <row r="259" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" s="15" t="s">
         <v>37</v>
       </c>
@@ -10115,7 +10105,7 @@
       <c r="J259" s="12"/>
       <c r="K259" s="12"/>
     </row>
-    <row r="260" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" s="15" t="s">
         <v>37</v>
       </c>
@@ -10136,7 +10126,7 @@
       <c r="J260" s="12"/>
       <c r="K260" s="12"/>
     </row>
-    <row r="261" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261" s="15" t="s">
         <v>37</v>
       </c>
@@ -10157,7 +10147,7 @@
       <c r="J261" s="12"/>
       <c r="K261" s="12"/>
     </row>
-    <row r="262" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" s="15" t="s">
         <v>37</v>
       </c>
@@ -10178,7 +10168,7 @@
       <c r="J262" s="12"/>
       <c r="K262" s="12"/>
     </row>
-    <row r="263" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A263" s="15" t="s">
         <v>37</v>
       </c>
@@ -10199,7 +10189,7 @@
       <c r="J263" s="12"/>
       <c r="K263" s="12"/>
     </row>
-    <row r="264" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264" s="15" t="s">
         <v>37</v>
       </c>
@@ -10220,7 +10210,7 @@
       <c r="J264" s="12"/>
       <c r="K264" s="12"/>
     </row>
-    <row r="265" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265" s="15" t="s">
         <v>37</v>
       </c>
@@ -10241,7 +10231,7 @@
       <c r="J265" s="12"/>
       <c r="K265" s="12"/>
     </row>
-    <row r="266" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" s="15" t="s">
         <v>37</v>
       </c>
@@ -10262,7 +10252,7 @@
       <c r="J266" s="12"/>
       <c r="K266" s="12"/>
     </row>
-    <row r="267" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267" s="15" t="s">
         <v>37</v>
       </c>
@@ -10283,7 +10273,7 @@
       <c r="J267" s="12"/>
       <c r="K267" s="12"/>
     </row>
-    <row r="268" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" s="15" t="s">
         <v>37</v>
       </c>
@@ -10304,7 +10294,7 @@
       <c r="J268" s="12"/>
       <c r="K268" s="12"/>
     </row>
-    <row r="269" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269" s="15" t="s">
         <v>37</v>
       </c>
@@ -10325,7 +10315,7 @@
       <c r="J269" s="12"/>
       <c r="K269" s="12"/>
     </row>
-    <row r="270" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A270" s="15" t="s">
         <v>37</v>
       </c>
@@ -10346,7 +10336,7 @@
       <c r="J270" s="12"/>
       <c r="K270" s="12"/>
     </row>
-    <row r="271" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271" s="15" t="s">
         <v>37</v>
       </c>
@@ -10367,7 +10357,7 @@
       <c r="J271" s="12"/>
       <c r="K271" s="12"/>
     </row>
-    <row r="272" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272" s="15" t="s">
         <v>37</v>
       </c>
@@ -10388,7 +10378,7 @@
       <c r="J272" s="12"/>
       <c r="K272" s="12"/>
     </row>
-    <row r="273" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273" s="15" t="s">
         <v>37</v>
       </c>
@@ -10409,7 +10399,7 @@
       <c r="J273" s="12"/>
       <c r="K273" s="12"/>
     </row>
-    <row r="274" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" s="15" t="s">
         <v>37</v>
       </c>
@@ -10430,7 +10420,7 @@
       <c r="J274" s="12"/>
       <c r="K274" s="12"/>
     </row>
-    <row r="275" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275" s="15" t="s">
         <v>37</v>
       </c>
@@ -10451,7 +10441,7 @@
       <c r="J275" s="12"/>
       <c r="K275" s="12"/>
     </row>
-    <row r="276" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A276" s="15" t="s">
         <v>37</v>
       </c>
@@ -10472,7 +10462,7 @@
       <c r="J276" s="12"/>
       <c r="K276" s="12"/>
     </row>
-    <row r="277" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277" s="15" t="s">
         <v>37</v>
       </c>
@@ -10493,7 +10483,7 @@
       <c r="J277" s="12"/>
       <c r="K277" s="12"/>
     </row>
-    <row r="278" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278" s="15" t="s">
         <v>37</v>
       </c>
@@ -10514,7 +10504,7 @@
       <c r="J278" s="12"/>
       <c r="K278" s="12"/>
     </row>
-    <row r="279" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A279" s="15" t="s">
         <v>37</v>
       </c>
@@ -10535,7 +10525,7 @@
       <c r="J279" s="12"/>
       <c r="K279" s="12"/>
     </row>
-    <row r="280" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A280" s="15" t="s">
         <v>37</v>
       </c>
@@ -10556,7 +10546,7 @@
       <c r="J280" s="12"/>
       <c r="K280" s="12"/>
     </row>
-    <row r="281" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A281" s="15" t="s">
         <v>37</v>
       </c>
@@ -10577,7 +10567,7 @@
       <c r="J281" s="12"/>
       <c r="K281" s="12"/>
     </row>
-    <row r="282" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A282" s="15" t="s">
         <v>37</v>
       </c>
@@ -10598,7 +10588,7 @@
       <c r="J282" s="12"/>
       <c r="K282" s="12"/>
     </row>
-    <row r="283" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A283" s="15" t="s">
         <v>37</v>
       </c>
@@ -10619,7 +10609,7 @@
       <c r="J283" s="12"/>
       <c r="K283" s="12"/>
     </row>
-    <row r="284" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A284" s="15" t="s">
         <v>37</v>
       </c>
@@ -10640,7 +10630,7 @@
       <c r="J284" s="12"/>
       <c r="K284" s="12"/>
     </row>
-    <row r="285" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A285" s="15" t="s">
         <v>37</v>
       </c>
@@ -10661,7 +10651,7 @@
       <c r="J285" s="12"/>
       <c r="K285" s="12"/>
     </row>
-    <row r="286" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A286" s="15" t="s">
         <v>37</v>
       </c>
@@ -10682,7 +10672,7 @@
       <c r="J286" s="12"/>
       <c r="K286" s="12"/>
     </row>
-    <row r="287" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A287" s="15" t="s">
         <v>37</v>
       </c>
@@ -10703,7 +10693,7 @@
       <c r="J287" s="12"/>
       <c r="K287" s="12"/>
     </row>
-    <row r="288" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A288" s="15" t="s">
         <v>37</v>
       </c>
@@ -10724,7 +10714,7 @@
       <c r="J288" s="12"/>
       <c r="K288" s="12"/>
     </row>
-    <row r="289" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A289" s="15" t="s">
         <v>37</v>
       </c>
@@ -10745,7 +10735,7 @@
       <c r="J289" s="12"/>
       <c r="K289" s="12"/>
     </row>
-    <row r="290" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A290" s="15" t="s">
         <v>37</v>
       </c>
@@ -10766,7 +10756,7 @@
       <c r="J290" s="12"/>
       <c r="K290" s="12"/>
     </row>
-    <row r="291" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A291" s="15" t="s">
         <v>37</v>
       </c>
@@ -10787,7 +10777,7 @@
       <c r="J291" s="12"/>
       <c r="K291" s="12"/>
     </row>
-    <row r="292" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A292" s="15" t="s">
         <v>37</v>
       </c>
@@ -10808,7 +10798,7 @@
       <c r="J292" s="12"/>
       <c r="K292" s="12"/>
     </row>
-    <row r="293" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A293" s="15" t="s">
         <v>37</v>
       </c>
@@ -10829,7 +10819,7 @@
       <c r="J293" s="12"/>
       <c r="K293" s="12"/>
     </row>
-    <row r="294" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A294" s="15" t="s">
         <v>37</v>
       </c>
@@ -10850,7 +10840,7 @@
       <c r="J294" s="12"/>
       <c r="K294" s="12"/>
     </row>
-    <row r="295" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A295" s="15" t="s">
         <v>37</v>
       </c>
@@ -10871,7 +10861,7 @@
       <c r="J295" s="12"/>
       <c r="K295" s="12"/>
     </row>
-    <row r="296" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A296" s="15" t="s">
         <v>37</v>
       </c>
@@ -10892,7 +10882,7 @@
       <c r="J296" s="12"/>
       <c r="K296" s="12"/>
     </row>
-    <row r="297" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A297" s="15" t="s">
         <v>37</v>
       </c>
@@ -10913,7 +10903,7 @@
       <c r="J297" s="12"/>
       <c r="K297" s="12"/>
     </row>
-    <row r="298" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298" s="15" t="s">
         <v>37</v>
       </c>
@@ -10934,7 +10924,7 @@
       <c r="J298" s="12"/>
       <c r="K298" s="12"/>
     </row>
-    <row r="299" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A299" s="15" t="s">
         <v>37</v>
       </c>
@@ -10955,7 +10945,7 @@
       <c r="J299" s="12"/>
       <c r="K299" s="12"/>
     </row>
-    <row r="300" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A300" s="15" t="s">
         <v>37</v>
       </c>
@@ -10976,7 +10966,7 @@
       <c r="J300" s="12"/>
       <c r="K300" s="12"/>
     </row>
-    <row r="301" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A301" s="15" t="s">
         <v>37</v>
       </c>
@@ -10997,7 +10987,7 @@
       <c r="J301" s="12"/>
       <c r="K301" s="12"/>
     </row>
-    <row r="302" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A302" s="15" t="s">
         <v>37</v>
       </c>
@@ -11018,7 +11008,7 @@
       <c r="J302" s="12"/>
       <c r="K302" s="12"/>
     </row>
-    <row r="303" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A303" s="15" t="s">
         <v>37</v>
       </c>
@@ -11039,7 +11029,7 @@
       <c r="J303" s="12"/>
       <c r="K303" s="12"/>
     </row>
-    <row r="304" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A304" s="15" t="s">
         <v>37</v>
       </c>
@@ -11060,7 +11050,7 @@
       <c r="J304" s="12"/>
       <c r="K304" s="12"/>
     </row>
-    <row r="305" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A305" s="15" t="s">
         <v>37</v>
       </c>
@@ -11081,7 +11071,7 @@
       <c r="J305" s="12"/>
       <c r="K305" s="12"/>
     </row>
-    <row r="306" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A306" s="15" t="s">
         <v>37</v>
       </c>
@@ -11102,7 +11092,7 @@
       <c r="J306" s="12"/>
       <c r="K306" s="12"/>
     </row>
-    <row r="307" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A307" s="15" t="s">
         <v>37</v>
       </c>
@@ -11123,7 +11113,7 @@
       <c r="J307" s="12"/>
       <c r="K307" s="12"/>
     </row>
-    <row r="308" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A308" s="15" t="s">
         <v>37</v>
       </c>
@@ -11144,7 +11134,7 @@
       <c r="J308" s="12"/>
       <c r="K308" s="12"/>
     </row>
-    <row r="309" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A309" s="15" t="s">
         <v>37</v>
       </c>
@@ -11165,7 +11155,7 @@
       <c r="J309" s="12"/>
       <c r="K309" s="12"/>
     </row>
-    <row r="310" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A310" s="15" t="s">
         <v>37</v>
       </c>
@@ -11186,7 +11176,7 @@
       <c r="J310" s="12"/>
       <c r="K310" s="12"/>
     </row>
-    <row r="311" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A311" s="15" t="s">
         <v>37</v>
       </c>
@@ -11207,7 +11197,7 @@
       <c r="J311" s="12"/>
       <c r="K311" s="12"/>
     </row>
-    <row r="312" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A312" s="15" t="s">
         <v>37</v>
       </c>
@@ -11228,7 +11218,7 @@
       <c r="J312" s="12"/>
       <c r="K312" s="12"/>
     </row>
-    <row r="313" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A313" s="15" t="s">
         <v>37</v>
       </c>
@@ -11249,7 +11239,7 @@
       <c r="J313" s="12"/>
       <c r="K313" s="12"/>
     </row>
-    <row r="314" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A314" s="15" t="s">
         <v>37</v>
       </c>
@@ -11270,7 +11260,7 @@
       <c r="J314" s="12"/>
       <c r="K314" s="12"/>
     </row>
-    <row r="315" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A315" s="15" t="s">
         <v>37</v>
       </c>
@@ -11291,7 +11281,7 @@
       <c r="J315" s="12"/>
       <c r="K315" s="12"/>
     </row>
-    <row r="316" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A316" s="15" t="s">
         <v>37</v>
       </c>
@@ -11312,7 +11302,7 @@
       <c r="J316" s="12"/>
       <c r="K316" s="12"/>
     </row>
-    <row r="317" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A317" s="15" t="s">
         <v>37</v>
       </c>
@@ -11333,7 +11323,7 @@
       <c r="J317" s="12"/>
       <c r="K317" s="12"/>
     </row>
-    <row r="318" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A318" s="15" t="s">
         <v>37</v>
       </c>
@@ -11354,7 +11344,7 @@
       <c r="J318" s="12"/>
       <c r="K318" s="12"/>
     </row>
-    <row r="319" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A319" s="15" t="s">
         <v>37</v>
       </c>
@@ -11375,7 +11365,7 @@
       <c r="J319" s="12"/>
       <c r="K319" s="12"/>
     </row>
-    <row r="320" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A320" s="15" t="s">
         <v>37</v>
       </c>
@@ -11396,7 +11386,7 @@
       <c r="J320" s="12"/>
       <c r="K320" s="12"/>
     </row>
-    <row r="321" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A321" s="5" t="s">
         <v>16</v>
       </c>
@@ -11423,7 +11413,7 @@
       <c r="J321" s="5"/>
       <c r="K321" s="5"/>
     </row>
-    <row r="322" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A322" s="5" t="s">
         <v>16</v>
       </c>
@@ -11450,7 +11440,7 @@
       <c r="J322" s="5"/>
       <c r="K322" s="5"/>
     </row>
-    <row r="323" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A323" s="5" t="s">
         <v>16</v>
       </c>
@@ -11479,7 +11469,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="324" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A324" s="5" t="s">
         <v>16</v>
       </c>
@@ -11508,7 +11498,7 @@
       </c>
       <c r="K324" s="37"/>
     </row>
-    <row r="325" spans="1:11" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A325" s="5" t="s">
         <v>12</v>
       </c>
@@ -11537,7 +11527,7 @@
       </c>
       <c r="K325" s="12"/>
     </row>
-    <row r="326" spans="1:11" customFormat="1" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A326" s="5" t="s">
         <v>12</v>
       </c>
@@ -11568,7 +11558,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="327" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A327" s="5" t="s">
         <v>16</v>
       </c>
@@ -11597,7 +11587,7 @@
       </c>
       <c r="K327" s="37"/>
     </row>
-    <row r="328" spans="1:11" customFormat="1" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:11" customFormat="1" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A328" s="5" t="s">
         <v>12</v>
       </c>
@@ -11626,7 +11616,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="329" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A329" s="15" t="s">
         <v>37</v>
       </c>
@@ -11647,7 +11637,7 @@
       <c r="J329" s="12"/>
       <c r="K329" s="12"/>
     </row>
-    <row r="330" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A330" s="15" t="s">
         <v>37</v>
       </c>
@@ -11668,7 +11658,7 @@
       <c r="J330" s="12"/>
       <c r="K330" s="12"/>
     </row>
-    <row r="331" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A331" s="15" t="s">
         <v>37</v>
       </c>
@@ -11689,7 +11679,7 @@
       <c r="J331" s="12"/>
       <c r="K331" s="12"/>
     </row>
-    <row r="332" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A332" s="15" t="s">
         <v>37</v>
       </c>
@@ -11710,7 +11700,7 @@
       <c r="J332" s="12"/>
       <c r="K332" s="12"/>
     </row>
-    <row r="333" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A333" s="15" t="s">
         <v>37</v>
       </c>
@@ -11731,7 +11721,7 @@
       <c r="J333" s="12"/>
       <c r="K333" s="12"/>
     </row>
-    <row r="334" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A334" s="15" t="s">
         <v>37</v>
       </c>
@@ -11752,7 +11742,7 @@
       <c r="J334" s="12"/>
       <c r="K334" s="12"/>
     </row>
-    <row r="335" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A335" s="15" t="s">
         <v>37</v>
       </c>
@@ -11773,7 +11763,7 @@
       <c r="J335" s="12"/>
       <c r="K335" s="12"/>
     </row>
-    <row r="336" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A336" s="15" t="s">
         <v>37</v>
       </c>
@@ -11794,7 +11784,7 @@
       <c r="J336" s="12"/>
       <c r="K336" s="12"/>
     </row>
-    <row r="337" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A337" s="15" t="s">
         <v>37</v>
       </c>
@@ -11815,7 +11805,7 @@
       <c r="J337" s="12"/>
       <c r="K337" s="12"/>
     </row>
-    <row r="338" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A338" s="15" t="s">
         <v>37</v>
       </c>
@@ -11836,7 +11826,7 @@
       <c r="J338" s="12"/>
       <c r="K338" s="12"/>
     </row>
-    <row r="339" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A339" s="15" t="s">
         <v>37</v>
       </c>
@@ -11857,7 +11847,7 @@
       <c r="J339" s="12"/>
       <c r="K339" s="12"/>
     </row>
-    <row r="340" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A340" s="15" t="s">
         <v>37</v>
       </c>
@@ -11878,7 +11868,7 @@
       <c r="J340" s="12"/>
       <c r="K340" s="12"/>
     </row>
-    <row r="341" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A341" s="5" t="s">
         <v>16</v>
       </c>
@@ -11907,7 +11897,7 @@
       </c>
       <c r="K341" s="37"/>
     </row>
-    <row r="342" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A342" s="5" t="s">
         <v>16</v>
       </c>
@@ -11934,7 +11924,7 @@
       <c r="J342" s="5"/>
       <c r="K342" s="5"/>
     </row>
-    <row r="343" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A343" s="5" t="s">
         <v>16</v>
       </c>
@@ -11959,7 +11949,7 @@
       <c r="J343" s="5"/>
       <c r="K343" s="5"/>
     </row>
-    <row r="344" spans="1:11" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A344" s="5" t="s">
         <v>12</v>
       </c>
@@ -11988,7 +11978,7 @@
       </c>
       <c r="K344" s="12"/>
     </row>
-    <row r="345" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A345" s="5" t="s">
         <v>16</v>
       </c>
@@ -12013,7 +12003,7 @@
       <c r="J345" s="5"/>
       <c r="K345" s="5"/>
     </row>
-    <row r="346" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A346" s="5" t="s">
         <v>16</v>
       </c>
@@ -12038,7 +12028,7 @@
       <c r="J346" s="5"/>
       <c r="K346" s="5"/>
     </row>
-    <row r="347" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A347" s="15" t="s">
         <v>37</v>
       </c>
@@ -12059,7 +12049,7 @@
       <c r="J347" s="12"/>
       <c r="K347" s="12"/>
     </row>
-    <row r="348" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A348" s="15" t="s">
         <v>37</v>
       </c>
@@ -12080,7 +12070,7 @@
       <c r="J348" s="12"/>
       <c r="K348" s="12"/>
     </row>
-    <row r="349" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="349" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A349" s="5" t="s">
         <v>16</v>
       </c>
@@ -12105,7 +12095,7 @@
       <c r="J349" s="5"/>
       <c r="K349" s="5"/>
     </row>
-    <row r="350" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A350" s="5" t="s">
         <v>16</v>
       </c>
@@ -12132,7 +12122,7 @@
       <c r="J350" s="5"/>
       <c r="K350" s="5"/>
     </row>
-    <row r="351" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A351" s="15" t="s">
         <v>37</v>
       </c>
@@ -12153,7 +12143,7 @@
       <c r="J351" s="12"/>
       <c r="K351" s="12"/>
     </row>
-    <row r="352" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A352" s="15" t="s">
         <v>37</v>
       </c>
@@ -12174,7 +12164,7 @@
       <c r="J352" s="12"/>
       <c r="K352" s="12"/>
     </row>
-    <row r="353" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A353" s="15" t="s">
         <v>37</v>
       </c>
@@ -12195,7 +12185,7 @@
       <c r="J353" s="12"/>
       <c r="K353" s="12"/>
     </row>
-    <row r="354" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A354" s="15" t="s">
         <v>37</v>
       </c>
@@ -12216,7 +12206,7 @@
       <c r="J354" s="12"/>
       <c r="K354" s="12"/>
     </row>
-    <row r="355" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A355" s="15" t="s">
         <v>37</v>
       </c>
@@ -12237,7 +12227,7 @@
       <c r="J355" s="12"/>
       <c r="K355" s="12"/>
     </row>
-    <row r="356" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A356" s="15" t="s">
         <v>37</v>
       </c>
@@ -12258,7 +12248,7 @@
       <c r="J356" s="12"/>
       <c r="K356" s="12"/>
     </row>
-    <row r="357" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A357" s="15" t="s">
         <v>37</v>
       </c>
@@ -12279,7 +12269,7 @@
       <c r="J357" s="12"/>
       <c r="K357" s="12"/>
     </row>
-    <row r="358" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A358" s="15" t="s">
         <v>37</v>
       </c>
@@ -12300,7 +12290,7 @@
       <c r="J358" s="12"/>
       <c r="K358" s="12"/>
     </row>
-    <row r="359" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A359" s="15" t="s">
         <v>37</v>
       </c>
@@ -12321,7 +12311,7 @@
       <c r="J359" s="12"/>
       <c r="K359" s="12"/>
     </row>
-    <row r="360" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A360" s="15" t="s">
         <v>37</v>
       </c>
@@ -12342,7 +12332,7 @@
       <c r="J360" s="12"/>
       <c r="K360" s="12"/>
     </row>
-    <row r="361" spans="1:11" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A361" s="5" t="s">
         <v>12</v>
       </c>
@@ -12371,7 +12361,7 @@
       </c>
       <c r="K361" s="12"/>
     </row>
-    <row r="362" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A362" s="15" t="s">
         <v>37</v>
       </c>
@@ -12392,7 +12382,7 @@
       <c r="J362" s="12"/>
       <c r="K362" s="12"/>
     </row>
-    <row r="363" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A363" s="15" t="s">
         <v>37</v>
       </c>
@@ -12413,7 +12403,7 @@
       <c r="J363" s="12"/>
       <c r="K363" s="12"/>
     </row>
-    <row r="364" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A364" s="15" t="s">
         <v>37</v>
       </c>
@@ -12434,7 +12424,7 @@
       <c r="J364" s="12"/>
       <c r="K364" s="12"/>
     </row>
-    <row r="365" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A365" s="15" t="s">
         <v>37</v>
       </c>
@@ -12455,7 +12445,7 @@
       <c r="J365" s="12"/>
       <c r="K365" s="12"/>
     </row>
-    <row r="366" spans="1:11" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A366" s="5" t="s">
         <v>12</v>
       </c>
@@ -12484,7 +12474,7 @@
       </c>
       <c r="K366" s="12"/>
     </row>
-    <row r="367" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A367" s="15" t="s">
         <v>37</v>
       </c>
@@ -12505,7 +12495,7 @@
       <c r="J367" s="12"/>
       <c r="K367" s="12"/>
     </row>
-    <row r="368" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A368" s="15" t="s">
         <v>37</v>
       </c>
@@ -12526,7 +12516,7 @@
       <c r="J368" s="12"/>
       <c r="K368" s="12"/>
     </row>
-    <row r="369" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A369" s="15" t="s">
         <v>37</v>
       </c>
@@ -12547,7 +12537,7 @@
       <c r="J369" s="12"/>
       <c r="K369" s="12"/>
     </row>
-    <row r="370" spans="1:11" customFormat="1" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A370" s="5" t="s">
         <v>12</v>
       </c>
@@ -12576,7 +12566,7 @@
       </c>
       <c r="K370" s="12"/>
     </row>
-    <row r="371" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A371" s="15" t="s">
         <v>37</v>
       </c>
@@ -12597,7 +12587,7 @@
       <c r="J371" s="12"/>
       <c r="K371" s="12"/>
     </row>
-    <row r="372" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A372" s="15" t="s">
         <v>37</v>
       </c>
@@ -12618,7 +12608,7 @@
       <c r="J372" s="12"/>
       <c r="K372" s="12"/>
     </row>
-    <row r="373" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A373" s="15" t="s">
         <v>37</v>
       </c>
@@ -12639,7 +12629,7 @@
       <c r="J373" s="12"/>
       <c r="K373" s="12"/>
     </row>
-    <row r="374" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A374" s="15" t="s">
         <v>37</v>
       </c>
@@ -12660,7 +12650,7 @@
       <c r="J374" s="12"/>
       <c r="K374" s="12"/>
     </row>
-    <row r="375" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A375" s="15" t="s">
         <v>37</v>
       </c>
@@ -12681,7 +12671,7 @@
       <c r="J375" s="12"/>
       <c r="K375" s="12"/>
     </row>
-    <row r="376" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A376" s="15" t="s">
         <v>37</v>
       </c>
@@ -12702,7 +12692,7 @@
       <c r="J376" s="12"/>
       <c r="K376" s="12"/>
     </row>
-    <row r="377" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A377" s="15" t="s">
         <v>37</v>
       </c>
@@ -12723,7 +12713,7 @@
       <c r="J377" s="12"/>
       <c r="K377" s="12"/>
     </row>
-    <row r="378" spans="1:11" customFormat="1" ht="25.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:11" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A378" s="15" t="s">
         <v>37</v>
       </c>
@@ -12744,7 +12734,7 @@
       <c r="J378" s="12"/>
       <c r="K378" s="12"/>
     </row>
-    <row r="379" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A379" s="15" t="s">
         <v>37</v>
       </c>
@@ -12765,7 +12755,7 @@
       <c r="J379" s="12"/>
       <c r="K379" s="12"/>
     </row>
-    <row r="380" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A380" s="15" t="s">
         <v>37</v>
       </c>
@@ -12786,7 +12776,7 @@
       <c r="J380" s="12"/>
       <c r="K380" s="12"/>
     </row>
-    <row r="381" spans="1:11" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A381" s="5" t="s">
         <v>12</v>
       </c>
@@ -12815,7 +12805,7 @@
       </c>
       <c r="K381" s="12"/>
     </row>
-    <row r="382" spans="1:11" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A382" s="5" t="s">
         <v>12</v>
       </c>
@@ -12844,7 +12834,7 @@
       </c>
       <c r="K382" s="12"/>
     </row>
-    <row r="383" spans="1:11" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:11" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A383" s="5" t="s">
         <v>12</v>
       </c>
@@ -12873,7 +12863,7 @@
       </c>
       <c r="K383" s="12"/>
     </row>
-    <row r="384" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A384" s="5" t="s">
         <v>881</v>
       </c>
@@ -12890,7 +12880,7 @@
       <c r="J384" s="12"/>
       <c r="K384" s="12"/>
     </row>
-    <row r="385" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A385" s="5" t="s">
         <v>881</v>
       </c>
@@ -12907,7 +12897,7 @@
       <c r="J385" s="12"/>
       <c r="K385" s="12"/>
     </row>
-    <row r="386" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A386" s="5" t="s">
         <v>881</v>
       </c>
@@ -12924,7 +12914,7 @@
       <c r="J386" s="12"/>
       <c r="K386" s="12"/>
     </row>
-    <row r="387" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A387" s="5" t="s">
         <v>881</v>
       </c>
@@ -12941,7 +12931,7 @@
       <c r="J387" s="12"/>
       <c r="K387" s="12"/>
     </row>
-    <row r="388" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A388" s="5" t="s">
         <v>881</v>
       </c>
@@ -12958,7 +12948,7 @@
       <c r="J388" s="12"/>
       <c r="K388" s="12"/>
     </row>
-    <row r="389" spans="1:11" s="3" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:11" s="3" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A389" s="5" t="s">
         <v>881</v>
       </c>
@@ -12975,7 +12965,7 @@
       <c r="J389" s="17"/>
       <c r="K389" s="17"/>
     </row>
-    <row r="390" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A390" s="5" t="s">
         <v>881</v>
       </c>
@@ -12992,7 +12982,7 @@
       <c r="J390" s="12"/>
       <c r="K390" s="12"/>
     </row>
-    <row r="391" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A391" s="5" t="s">
         <v>881</v>
       </c>
@@ -13009,7 +12999,7 @@
       <c r="J391" s="12"/>
       <c r="K391" s="12"/>
     </row>
-    <row r="392" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A392" s="5" t="s">
         <v>881</v>
       </c>
@@ -13026,7 +13016,7 @@
       <c r="J392" s="12"/>
       <c r="K392" s="12"/>
     </row>
-    <row r="393" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A393" s="5" t="s">
         <v>881</v>
       </c>
@@ -13043,7 +13033,7 @@
       <c r="J393" s="12"/>
       <c r="K393" s="12"/>
     </row>
-    <row r="394" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A394" s="5" t="s">
         <v>881</v>
       </c>
@@ -13060,7 +13050,7 @@
       <c r="J394" s="12"/>
       <c r="K394" s="12"/>
     </row>
-    <row r="395" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A395" s="5" t="s">
         <v>881</v>
       </c>
@@ -13077,7 +13067,7 @@
       <c r="J395" s="12"/>
       <c r="K395" s="12"/>
     </row>
-    <row r="396" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A396" s="5" t="s">
         <v>881</v>
       </c>
@@ -13094,7 +13084,7 @@
       <c r="J396" s="12"/>
       <c r="K396" s="12"/>
     </row>
-    <row r="397" spans="1:11" s="3" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:11" s="3" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A397" s="5" t="s">
         <v>881</v>
       </c>
@@ -13111,7 +13101,7 @@
       <c r="J397" s="17"/>
       <c r="K397" s="17"/>
     </row>
-    <row r="398" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A398" s="5" t="s">
         <v>881</v>
       </c>
@@ -13128,7 +13118,7 @@
       <c r="J398" s="12"/>
       <c r="K398" s="12"/>
     </row>
-    <row r="399" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A399" s="5" t="s">
         <v>881</v>
       </c>
@@ -13145,7 +13135,7 @@
       <c r="J399" s="12"/>
       <c r="K399" s="12"/>
     </row>
-    <row r="400" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A400" s="5" t="s">
         <v>881</v>
       </c>
@@ -13162,7 +13152,7 @@
       <c r="J400" s="12"/>
       <c r="K400" s="12"/>
     </row>
-    <row r="401" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A401" s="5" t="s">
         <v>881</v>
       </c>
@@ -13179,7 +13169,7 @@
       <c r="J401" s="12"/>
       <c r="K401" s="12"/>
     </row>
-    <row r="402" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A402" s="5" t="s">
         <v>881</v>
       </c>
@@ -13196,7 +13186,7 @@
       <c r="J402" s="12"/>
       <c r="K402" s="12"/>
     </row>
-    <row r="403" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="403" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A403" s="5" t="s">
         <v>16</v>
       </c>
@@ -13225,7 +13215,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="404" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="404" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A404" s="5" t="s">
         <v>16</v>
       </c>
@@ -13254,7 +13244,7 @@
       </c>
       <c r="K404" s="5"/>
     </row>
-    <row r="405" spans="1:11" s="38" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="405" spans="1:11" s="38" customFormat="1" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A405" s="5" t="s">
         <v>16</v>
       </c>
@@ -13283,7 +13273,7 @@
       </c>
       <c r="K405" s="37"/>
     </row>
-    <row r="406" spans="1:11" s="38" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="406" spans="1:11" s="38" customFormat="1" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A406" s="5" t="s">
         <v>16</v>
       </c>
@@ -13310,7 +13300,7 @@
       <c r="J406" s="37"/>
       <c r="K406" s="37"/>
     </row>
-    <row r="407" spans="1:11" s="3" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:11" s="3" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A407" s="5" t="s">
         <v>881</v>
       </c>
@@ -13327,7 +13317,7 @@
       <c r="J407" s="17"/>
       <c r="K407" s="17"/>
     </row>
-    <row r="408" spans="1:11" s="3" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:11" s="3" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A408" s="5" t="s">
         <v>881</v>
       </c>
@@ -13344,7 +13334,7 @@
       <c r="J408" s="17"/>
       <c r="K408" s="17"/>
     </row>
-    <row r="409" spans="1:11" s="3" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:11" s="3" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A409" s="5" t="s">
         <v>881</v>
       </c>
@@ -13361,7 +13351,7 @@
       <c r="J409" s="17"/>
       <c r="K409" s="17"/>
     </row>
-    <row r="410" spans="1:11" s="3" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:11" s="3" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A410" s="5" t="s">
         <v>881</v>
       </c>
@@ -13378,7 +13368,7 @@
       <c r="J410" s="17"/>
       <c r="K410" s="17"/>
     </row>
-    <row r="411" spans="1:11" s="3" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:11" s="3" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A411" s="5" t="s">
         <v>881</v>
       </c>
@@ -13395,7 +13385,7 @@
       <c r="J411" s="17"/>
       <c r="K411" s="17"/>
     </row>
-    <row r="412" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A412" s="5" t="s">
         <v>881</v>
       </c>
@@ -13412,7 +13402,7 @@
       <c r="J412" s="12"/>
       <c r="K412" s="12"/>
     </row>
-    <row r="413" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A413" s="5" t="s">
         <v>881</v>
       </c>
@@ -13429,7 +13419,7 @@
       <c r="J413" s="12"/>
       <c r="K413" s="12"/>
     </row>
-    <row r="414" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A414" s="5" t="s">
         <v>881</v>
       </c>
@@ -13446,7 +13436,7 @@
       <c r="J414" s="12"/>
       <c r="K414" s="12"/>
     </row>
-    <row r="415" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A415" s="5" t="s">
         <v>881</v>
       </c>
@@ -13463,7 +13453,7 @@
       <c r="J415" s="12"/>
       <c r="K415" s="12"/>
     </row>
-    <row r="416" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A416" s="5" t="s">
         <v>881</v>
       </c>
@@ -13480,7 +13470,7 @@
       <c r="J416" s="12"/>
       <c r="K416" s="12"/>
     </row>
-    <row r="417" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A417" s="5" t="s">
         <v>881</v>
       </c>
@@ -13497,7 +13487,7 @@
       <c r="J417" s="12"/>
       <c r="K417" s="12"/>
     </row>
-    <row r="418" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A418" s="5" t="s">
         <v>881</v>
       </c>
@@ -13514,7 +13504,7 @@
       <c r="J418" s="12"/>
       <c r="K418" s="12"/>
     </row>
-    <row r="419" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A419" s="5" t="s">
         <v>881</v>
       </c>
@@ -13531,7 +13521,7 @@
       <c r="J419" s="12"/>
       <c r="K419" s="12"/>
     </row>
-    <row r="420" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A420" s="5" t="s">
         <v>881</v>
       </c>
@@ -13548,7 +13538,7 @@
       <c r="J420" s="12"/>
       <c r="K420" s="12"/>
     </row>
-    <row r="421" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A421" s="5" t="s">
         <v>881</v>
       </c>
@@ -13565,7 +13555,7 @@
       <c r="J421" s="12"/>
       <c r="K421" s="12"/>
     </row>
-    <row r="422" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A422" s="5" t="s">
         <v>881</v>
       </c>
@@ -13582,7 +13572,7 @@
       <c r="J422" s="12"/>
       <c r="K422" s="12"/>
     </row>
-    <row r="423" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A423" s="5" t="s">
         <v>881</v>
       </c>
@@ -13599,7 +13589,7 @@
       <c r="J423" s="12"/>
       <c r="K423" s="12"/>
     </row>
-    <row r="424" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A424" s="5" t="s">
         <v>881</v>
       </c>
@@ -13616,7 +13606,7 @@
       <c r="J424" s="12"/>
       <c r="K424" s="12"/>
     </row>
-    <row r="425" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A425" s="5" t="s">
         <v>881</v>
       </c>
@@ -13633,7 +13623,7 @@
       <c r="J425" s="12"/>
       <c r="K425" s="12"/>
     </row>
-    <row r="426" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A426" s="5" t="s">
         <v>881</v>
       </c>
@@ -13650,7 +13640,7 @@
       <c r="J426" s="12"/>
       <c r="K426" s="12"/>
     </row>
-    <row r="427" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A427" s="5" t="s">
         <v>881</v>
       </c>
@@ -13667,7 +13657,7 @@
       <c r="J427" s="12"/>
       <c r="K427" s="12"/>
     </row>
-    <row r="428" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A428" s="5" t="s">
         <v>881</v>
       </c>
@@ -13684,7 +13674,7 @@
       <c r="J428" s="12"/>
       <c r="K428" s="12"/>
     </row>
-    <row r="429" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A429" s="5" t="s">
         <v>881</v>
       </c>
@@ -13701,7 +13691,7 @@
       <c r="J429" s="12"/>
       <c r="K429" s="12"/>
     </row>
-    <row r="430" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A430" s="5" t="s">
         <v>881</v>
       </c>
@@ -13718,7 +13708,7 @@
       <c r="J430" s="12"/>
       <c r="K430" s="12"/>
     </row>
-    <row r="431" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A431" s="5" t="s">
         <v>881</v>
       </c>
@@ -13735,7 +13725,7 @@
       <c r="J431" s="12"/>
       <c r="K431" s="12"/>
     </row>
-    <row r="432" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A432" s="5" t="s">
         <v>881</v>
       </c>
@@ -13752,7 +13742,7 @@
       <c r="J432" s="12"/>
       <c r="K432" s="12"/>
     </row>
-    <row r="433" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A433" s="5" t="s">
         <v>881</v>
       </c>
@@ -13769,7 +13759,7 @@
       <c r="J433" s="12"/>
       <c r="K433" s="12"/>
     </row>
-    <row r="434" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A434" s="5" t="s">
         <v>881</v>
       </c>
@@ -13786,7 +13776,7 @@
       <c r="J434" s="12"/>
       <c r="K434" s="12"/>
     </row>
-    <row r="435" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A435" s="5" t="s">
         <v>881</v>
       </c>
@@ -13803,7 +13793,7 @@
       <c r="J435" s="12"/>
       <c r="K435" s="12"/>
     </row>
-    <row r="436" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A436" s="5" t="s">
         <v>881</v>
       </c>
@@ -13820,7 +13810,7 @@
       <c r="J436" s="12"/>
       <c r="K436" s="12"/>
     </row>
-    <row r="437" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A437" s="5" t="s">
         <v>881</v>
       </c>
@@ -13837,7 +13827,7 @@
       <c r="J437" s="12"/>
       <c r="K437" s="12"/>
     </row>
-    <row r="438" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A438" s="5" t="s">
         <v>881</v>
       </c>
@@ -13854,7 +13844,7 @@
       <c r="J438" s="12"/>
       <c r="K438" s="12"/>
     </row>
-    <row r="439" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A439" s="5" t="s">
         <v>881</v>
       </c>
@@ -13871,7 +13861,7 @@
       <c r="J439" s="12"/>
       <c r="K439" s="12"/>
     </row>
-    <row r="440" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A440" s="5" t="s">
         <v>881</v>
       </c>
@@ -13888,7 +13878,7 @@
       <c r="J440" s="12"/>
       <c r="K440" s="12"/>
     </row>
-    <row r="441" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A441" s="5" t="s">
         <v>881</v>
       </c>
@@ -13905,7 +13895,7 @@
       <c r="J441" s="12"/>
       <c r="K441" s="12"/>
     </row>
-    <row r="442" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A442" s="5" t="s">
         <v>881</v>
       </c>
@@ -13922,7 +13912,7 @@
       <c r="J442" s="12"/>
       <c r="K442" s="12"/>
     </row>
-    <row r="443" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A443" s="5" t="s">
         <v>881</v>
       </c>
@@ -13939,7 +13929,7 @@
       <c r="J443" s="12"/>
       <c r="K443" s="12"/>
     </row>
-    <row r="444" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A444" s="5" t="s">
         <v>881</v>
       </c>
@@ -13956,7 +13946,7 @@
       <c r="J444" s="12"/>
       <c r="K444" s="12"/>
     </row>
-    <row r="445" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A445" s="5" t="s">
         <v>881</v>
       </c>
@@ -13973,7 +13963,7 @@
       <c r="J445" s="12"/>
       <c r="K445" s="12"/>
     </row>
-    <row r="446" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A446" s="5" t="s">
         <v>881</v>
       </c>
@@ -13990,7 +13980,7 @@
       <c r="J446" s="12"/>
       <c r="K446" s="12"/>
     </row>
-    <row r="447" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="447" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A447" s="5" t="s">
         <v>881</v>
       </c>
@@ -14007,7 +13997,7 @@
       <c r="J447" s="12"/>
       <c r="K447" s="12"/>
     </row>
-    <row r="448" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A448" s="5" t="s">
         <v>881</v>
       </c>
@@ -14024,7 +14014,7 @@
       <c r="J448" s="12"/>
       <c r="K448" s="12"/>
     </row>
-    <row r="449" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A449" s="5" t="s">
         <v>881</v>
       </c>
@@ -14041,7 +14031,7 @@
       <c r="J449" s="12"/>
       <c r="K449" s="12"/>
     </row>
-    <row r="450" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A450" s="5" t="s">
         <v>881</v>
       </c>
@@ -14058,7 +14048,7 @@
       <c r="J450" s="12"/>
       <c r="K450" s="12"/>
     </row>
-    <row r="451" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A451" s="5" t="s">
         <v>881</v>
       </c>
@@ -14075,7 +14065,7 @@
       <c r="J451" s="12"/>
       <c r="K451" s="12"/>
     </row>
-    <row r="452" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A452" s="5" t="s">
         <v>881</v>
       </c>
@@ -14092,7 +14082,7 @@
       <c r="J452" s="12"/>
       <c r="K452" s="12"/>
     </row>
-    <row r="453" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A453" s="5" t="s">
         <v>881</v>
       </c>
@@ -14109,7 +14099,7 @@
       <c r="J453" s="12"/>
       <c r="K453" s="12"/>
     </row>
-    <row r="454" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A454" s="5" t="s">
         <v>881</v>
       </c>
@@ -14126,7 +14116,7 @@
       <c r="J454" s="12"/>
       <c r="K454" s="12"/>
     </row>
-    <row r="455" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A455" s="5" t="s">
         <v>881</v>
       </c>
@@ -14143,7 +14133,7 @@
       <c r="J455" s="12"/>
       <c r="K455" s="12"/>
     </row>
-    <row r="456" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A456" s="5" t="s">
         <v>881</v>
       </c>
@@ -14160,7 +14150,7 @@
       <c r="J456" s="12"/>
       <c r="K456" s="12"/>
     </row>
-    <row r="457" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A457" s="5" t="s">
         <v>881</v>
       </c>
@@ -14177,7 +14167,7 @@
       <c r="J457" s="12"/>
       <c r="K457" s="12"/>
     </row>
-    <row r="458" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A458" s="5" t="s">
         <v>881</v>
       </c>
@@ -14194,7 +14184,7 @@
       <c r="J458" s="12"/>
       <c r="K458" s="12"/>
     </row>
-    <row r="459" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A459" s="5" t="s">
         <v>881</v>
       </c>
@@ -14211,7 +14201,7 @@
       <c r="J459" s="12"/>
       <c r="K459" s="12"/>
     </row>
-    <row r="460" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="460" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A460" s="5" t="s">
         <v>881</v>
       </c>
@@ -14228,7 +14218,7 @@
       <c r="J460" s="12"/>
       <c r="K460" s="12"/>
     </row>
-    <row r="461" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A461" s="5" t="s">
         <v>881</v>
       </c>
@@ -14245,7 +14235,7 @@
       <c r="J461" s="12"/>
       <c r="K461" s="12"/>
     </row>
-    <row r="462" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A462" s="5" t="s">
         <v>881</v>
       </c>
@@ -14262,7 +14252,7 @@
       <c r="J462" s="12"/>
       <c r="K462" s="12"/>
     </row>
-    <row r="463" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A463" s="5" t="s">
         <v>881</v>
       </c>
@@ -14279,7 +14269,7 @@
       <c r="J463" s="12"/>
       <c r="K463" s="12"/>
     </row>
-    <row r="464" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A464" s="5" t="s">
         <v>881</v>
       </c>
@@ -14296,7 +14286,7 @@
       <c r="J464" s="12"/>
       <c r="K464" s="12"/>
     </row>
-    <row r="465" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="465" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A465" s="5" t="s">
         <v>881</v>
       </c>
@@ -14313,7 +14303,7 @@
       <c r="J465" s="12"/>
       <c r="K465" s="12"/>
     </row>
-    <row r="466" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A466" s="5" t="s">
         <v>881</v>
       </c>
@@ -14330,7 +14320,7 @@
       <c r="J466" s="12"/>
       <c r="K466" s="12"/>
     </row>
-    <row r="467" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A467" s="5" t="s">
         <v>881</v>
       </c>
@@ -14347,7 +14337,7 @@
       <c r="J467" s="12"/>
       <c r="K467" s="12"/>
     </row>
-    <row r="468" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="468" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A468" s="5" t="s">
         <v>881</v>
       </c>
@@ -14364,7 +14354,7 @@
       <c r="J468" s="12"/>
       <c r="K468" s="12"/>
     </row>
-    <row r="469" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="469" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A469" s="5" t="s">
         <v>881</v>
       </c>
@@ -14381,7 +14371,7 @@
       <c r="J469" s="12"/>
       <c r="K469" s="12"/>
     </row>
-    <row r="470" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A470" s="5" t="s">
         <v>881</v>
       </c>
@@ -14398,7 +14388,7 @@
       <c r="J470" s="12"/>
       <c r="K470" s="12"/>
     </row>
-    <row r="471" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A471" s="5" t="s">
         <v>881</v>
       </c>
@@ -14415,7 +14405,7 @@
       <c r="J471" s="12"/>
       <c r="K471" s="12"/>
     </row>
-    <row r="472" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A472" s="5" t="s">
         <v>881</v>
       </c>
@@ -14432,7 +14422,7 @@
       <c r="J472" s="12"/>
       <c r="K472" s="12"/>
     </row>
-    <row r="473" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A473" s="5" t="s">
         <v>881</v>
       </c>
@@ -14449,7 +14439,7 @@
       <c r="J473" s="12"/>
       <c r="K473" s="12"/>
     </row>
-    <row r="474" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A474" s="5" t="s">
         <v>881</v>
       </c>
@@ -14466,7 +14456,7 @@
       <c r="J474" s="12"/>
       <c r="K474" s="12"/>
     </row>
-    <row r="475" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="475" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A475" s="5" t="s">
         <v>881</v>
       </c>
@@ -14483,7 +14473,7 @@
       <c r="J475" s="12"/>
       <c r="K475" s="12"/>
     </row>
-    <row r="476" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A476" s="5" t="s">
         <v>881</v>
       </c>
@@ -14500,7 +14490,7 @@
       <c r="J476" s="12"/>
       <c r="K476" s="12"/>
     </row>
-    <row r="477" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A477" s="5" t="s">
         <v>881</v>
       </c>
@@ -14517,7 +14507,7 @@
       <c r="J477" s="12"/>
       <c r="K477" s="12"/>
     </row>
-    <row r="478" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A478" s="5" t="s">
         <v>881</v>
       </c>
@@ -14534,7 +14524,7 @@
       <c r="J478" s="12"/>
       <c r="K478" s="12"/>
     </row>
-    <row r="479" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A479" s="5" t="s">
         <v>881</v>
       </c>
@@ -14551,7 +14541,7 @@
       <c r="J479" s="12"/>
       <c r="K479" s="12"/>
     </row>
-    <row r="480" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A480" s="5" t="s">
         <v>881</v>
       </c>
@@ -14568,7 +14558,7 @@
       <c r="J480" s="12"/>
       <c r="K480" s="12"/>
     </row>
-    <row r="481" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A481" s="5" t="s">
         <v>881</v>
       </c>
@@ -14585,7 +14575,7 @@
       <c r="J481" s="12"/>
       <c r="K481" s="12"/>
     </row>
-    <row r="482" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A482" s="5" t="s">
         <v>881</v>
       </c>
@@ -14602,7 +14592,7 @@
       <c r="J482" s="12"/>
       <c r="K482" s="12"/>
     </row>
-    <row r="483" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="483" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A483" s="5" t="s">
         <v>881</v>
       </c>
@@ -14619,7 +14609,7 @@
       <c r="J483" s="12"/>
       <c r="K483" s="12"/>
     </row>
-    <row r="484" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="484" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A484" s="5" t="s">
         <v>881</v>
       </c>
@@ -14636,7 +14626,7 @@
       <c r="J484" s="12"/>
       <c r="K484" s="12"/>
     </row>
-    <row r="485" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="485" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A485" s="5" t="s">
         <v>881</v>
       </c>
@@ -14653,7 +14643,7 @@
       <c r="J485" s="12"/>
       <c r="K485" s="12"/>
     </row>
-    <row r="486" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="486" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A486" s="5" t="s">
         <v>881</v>
       </c>
@@ -14670,7 +14660,7 @@
       <c r="J486" s="12"/>
       <c r="K486" s="12"/>
     </row>
-    <row r="487" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="487" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A487" s="5" t="s">
         <v>881</v>
       </c>
@@ -14687,7 +14677,7 @@
       <c r="J487" s="12"/>
       <c r="K487" s="12"/>
     </row>
-    <row r="488" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="488" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A488" s="5" t="s">
         <v>881</v>
       </c>
@@ -14704,7 +14694,7 @@
       <c r="J488" s="12"/>
       <c r="K488" s="12"/>
     </row>
-    <row r="489" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="489" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A489" s="5" t="s">
         <v>881</v>
       </c>
@@ -14721,7 +14711,7 @@
       <c r="J489" s="12"/>
       <c r="K489" s="12"/>
     </row>
-    <row r="490" spans="1:11" customFormat="1" ht="15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="490" spans="1:11" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A490" s="5" t="s">
         <v>881</v>
       </c>
@@ -14738,7 +14728,7 @@
       <c r="J490" s="12"/>
       <c r="K490" s="12"/>
     </row>
-    <row r="491" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="491" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A491" s="5" t="s">
         <v>16</v>
       </c>
@@ -14765,7 +14755,7 @@
       <c r="J491" s="37"/>
       <c r="K491" s="37"/>
     </row>
-    <row r="492" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="492" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A492" s="5" t="s">
         <v>16</v>
       </c>
@@ -14792,7 +14782,7 @@
       <c r="J492" s="37"/>
       <c r="K492" s="37"/>
     </row>
-    <row r="493" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="493" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A493" s="5" t="s">
         <v>16</v>
       </c>
@@ -14819,7 +14809,7 @@
       <c r="J493" s="37"/>
       <c r="K493" s="37"/>
     </row>
-    <row r="494" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="494" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A494" s="5" t="s">
         <v>16</v>
       </c>
@@ -14846,7 +14836,7 @@
       <c r="J494" s="37"/>
       <c r="K494" s="37"/>
     </row>
-    <row r="495" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="495" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A495" s="5" t="s">
         <v>16</v>
       </c>
@@ -14873,7 +14863,7 @@
       <c r="J495" s="37"/>
       <c r="K495" s="37"/>
     </row>
-    <row r="496" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="496" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A496" s="5" t="s">
         <v>16</v>
       </c>
@@ -14900,7 +14890,7 @@
       <c r="J496" s="37"/>
       <c r="K496" s="37"/>
     </row>
-    <row r="497" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="497" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A497" s="5" t="s">
         <v>16</v>
       </c>
@@ -14927,7 +14917,7 @@
       <c r="J497" s="37"/>
       <c r="K497" s="37"/>
     </row>
-    <row r="498" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="498" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A498" s="5" t="s">
         <v>16</v>
       </c>
@@ -14954,7 +14944,7 @@
       <c r="J498" s="37"/>
       <c r="K498" s="37"/>
     </row>
-    <row r="499" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="499" spans="1:11" ht="41.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A499" s="5" t="s">
         <v>16</v>
       </c>
@@ -14981,7 +14971,7 @@
       <c r="J499" s="37"/>
       <c r="K499" s="37"/>
     </row>
-    <row r="500" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="500" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A500" s="5" t="s">
         <v>16</v>
       </c>
@@ -15006,7 +14996,7 @@
       <c r="J500" s="5"/>
       <c r="K500" s="5"/>
     </row>
-    <row r="501" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="501" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A501" s="5" t="s">
         <v>16</v>
       </c>
@@ -15033,7 +15023,7 @@
       </c>
       <c r="K501" s="5"/>
     </row>
-    <row r="502" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="502" spans="1:11" ht="69" hidden="1" x14ac:dyDescent="0.3">
       <c r="A502" s="5" t="s">
         <v>16</v>
       </c>
@@ -15062,7 +15052,7 @@
         <v>1020</v>
       </c>
     </row>
-    <row r="503" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="503" spans="1:11" ht="27.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A503" s="5" t="s">
         <v>16</v>
       </c>
@@ -15087,7 +15077,7 @@
       </c>
       <c r="K503" s="5"/>
     </row>
-    <row r="504" spans="1:11" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="504" spans="1:11" ht="82.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A504" s="5" t="s">
         <v>16</v>
       </c>
@@ -15122,6 +15112,11 @@
       <filters>
         <filter val="DEET"/>
         <filter val="Navigator/DEET"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Reefer Configuration"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K504">

</xml_diff>